<commit_message>
Radically simplify Capital Gains Tax Calculator
Replaced the previous version (sale-scenario lot table, before/after
comparison, tax-loss-harvesting what-if) with a single, direct flow:
Your Info -> Capital Gains & Losses -> Estimated Tax. One screen, one
answer. The tax shown is specifically the tax generated by the entered
gains/losses (short-term gain taxed incrementally at ordinary rates,
long-term gain stacked at preferential rates, NIIT, state), not the
household's total tax bill.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XveA8LngnD1MFNqnzekQW3
</commit_message>
<xml_diff>
--- a/Capital_Gains_Tax_Estimator.xlsx
+++ b/Capital_Gains_Tax_Estimator.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Capital Gains Tax Estimator" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Capital Gains Tax Calculator" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Tax Rates &amp; Assumptions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$#,##0;($#,##0)"/>
   </numFmts>
-  <fonts count="33">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,24 +99,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
@@ -127,26 +109,14 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
@@ -185,23 +155,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="10"/>
@@ -210,10 +163,16 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3864"/>
-      <sz val="14"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -250,14 +209,8 @@
         <bgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -279,44 +232,11 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -360,104 +280,61 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="32" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="10" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="165" fontId="24" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="164" fontId="24" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="31" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="165" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,7 +423,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Estimated Tax From Sale - By Type</a:t>
+              <a:t>Estimated Tax - By Type</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -560,7 +437,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Capital Gains Tax Estimator'!G69</f>
+              <f>'Capital Gains Tax Calculator'!G36</f>
             </strRef>
           </tx>
           <spPr>
@@ -570,12 +447,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Capital Gains Tax Estimator'!$F$70:$F$72</f>
+              <f>'Capital Gains Tax Calculator'!$F$37:$F$39</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capital Gains Tax Estimator'!$G$70:$G$72</f>
+              <f>'Capital Gains Tax Calculator'!$G$37:$G$39</f>
             </numRef>
           </val>
         </ser>
@@ -600,7 +477,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>68</row>
+      <row>35</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2700000"/>
@@ -910,17 +787,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N176"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:N95"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
@@ -932,2072 +808,1055 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>CAPITAL GAINS &amp; LOSSES TAX ESTIMATOR</t>
+          <t>CAPITAL GAINS TAX CALCULATOR</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="20" t="inlineStr">
         <is>
-          <t>Estimate the tax impact of selling an investment. For planning purposes only - not tax, legal, or accounting advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
-        <is>
-          <t>ESTIMATED TAX FROM PORTFOLIO SALE</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="B5" s="22" t="inlineStr">
+          <t>Estimated tax from capital gains and losses. For planning purposes only - not tax, legal, or accounting advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>YOUR INFO</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Tax Year</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Filing Status</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Married Filing Jointly</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>State of Residence</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>State Tax Rate if 'Other (Manual Entry)' Selected</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Taxable Income (before these gains/losses)</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>(your salary/other income after deductions - used only to determine which tax brackets your gains fall into)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>CAPITAL GAINS &amp; LOSSES</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Short-Term Capital Gains (held 1 year or less)</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Long-Term Capital Gains (held more than 1 year)</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>155000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>Short-Term Capital Losses</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Long-Term Capital Losses</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Capital Loss Carryforward (from prior years)</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>ESTIMATED TAX</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>Total Estimated Tax</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="inlineStr">
         <is>
           <t>Federal Tax</t>
         </is>
       </c>
-      <c r="C5" s="22" t="inlineStr">
+      <c r="E20" s="25" t="inlineStr">
         <is>
           <t>State Tax</t>
         </is>
       </c>
-      <c r="D5" s="22" t="inlineStr">
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="38">
+        <f>C80</f>
+        <v/>
+      </c>
+      <c r="C21" s="39">
+        <f>C81</f>
+        <v/>
+      </c>
+      <c r="D21" s="38">
+        <f>(C73+C74)</f>
+        <v/>
+      </c>
+      <c r="E21" s="38">
+        <f>C79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Net Short-Term Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C23" s="40">
+        <f>C64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>Net Long-Term Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C24" s="40">
+        <f>C65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Total Net Capital Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C25" s="41">
+        <f>C66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Capital Loss Deduction (against ordinary income)</t>
+        </is>
+      </c>
+      <c r="C26" s="40">
+        <f>IF(C66&lt;0,MAX(C66,-C60),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Capital Loss Carryforward to Future Years</t>
+        </is>
+      </c>
+      <c r="C27" s="40">
+        <f>-C69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>Federal Tax on Short-Term Gain (ordinary rates)</t>
+        </is>
+      </c>
+      <c r="C28" s="40">
+        <f>C73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Federal Tax on Long-Term Gain (preferential rates)</t>
+        </is>
+      </c>
+      <c r="C29" s="40">
+        <f>C74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>Net Investment Income Tax (NIIT)</t>
+        </is>
+      </c>
+      <c r="C30" s="40">
+        <f>C77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>State Tax</t>
+        </is>
+      </c>
+      <c r="C31" s="40">
+        <f>C79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Total Estimated Tax</t>
+        </is>
+      </c>
+      <c r="C32" s="41">
+        <f>C80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate on the Gain</t>
+        </is>
+      </c>
+      <c r="C33" s="42">
+        <f>C81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="24" t="inlineStr">
+        <is>
+          <t>Marginal Long-Term Capital Gains Rate</t>
+        </is>
+      </c>
+      <c r="C34" s="42">
+        <f>C82</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Tax Component</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="F37" s="28" t="inlineStr">
+        <is>
+          <t>Federal Tax</t>
+        </is>
+      </c>
+      <c r="G37" s="43">
+        <f>(C73+C74)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="F38" s="28" t="inlineStr">
+        <is>
+          <t>State Tax</t>
+        </is>
+      </c>
+      <c r="G38" s="43">
+        <f>C79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="F39" s="28" t="inlineStr">
         <is>
           <t>NIIT</t>
         </is>
       </c>
-      <c r="E5" s="22" t="inlineStr">
+      <c r="G39" s="43">
+        <f>C77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="26" t="inlineStr">
+        <is>
+          <t>Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="57" hidden="1" outlineLevel="1" collapsed="1">
+      <c r="A57" s="27" t="inlineStr">
+        <is>
+          <t>CALCULATION DETAIL (grouped - click + to expand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" hidden="1" outlineLevel="1"/>
+    <row r="59" hidden="1" outlineLevel="1">
+      <c r="B59" s="32" t="inlineStr">
+        <is>
+          <t>Standard Deduction (add-back for MAGI estimate)</t>
+        </is>
+      </c>
+      <c r="C59" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L65)</f>
+        <v/>
+      </c>
+      <c r="K59" s="7" t="inlineStr">
+        <is>
+          <t>Filing Status</t>
+        </is>
+      </c>
+      <c r="L59" s="28">
+        <f>C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" hidden="1" outlineLevel="1">
+      <c r="B60" s="32" t="inlineStr">
+        <is>
+          <t>Capital Loss Limit vs. Ordinary Income</t>
+        </is>
+      </c>
+      <c r="C60" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L64)</f>
+        <v/>
+      </c>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>Tax Year</t>
+        </is>
+      </c>
+      <c r="L60" s="28">
+        <f>C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" hidden="1" outlineLevel="1">
+      <c r="B61" s="32" t="inlineStr">
+        <is>
+          <t>NIIT Threshold</t>
+        </is>
+      </c>
+      <c r="C61" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L64)</f>
+        <v/>
+      </c>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>Federal Key</t>
+        </is>
+      </c>
+      <c r="L61" s="28">
+        <f>L60&amp;"|"&amp;L59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" hidden="1" outlineLevel="1">
+      <c r="B62" s="32" t="inlineStr">
+        <is>
+          <t>NIIT Rate</t>
+        </is>
+      </c>
+      <c r="C62" s="34">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L64)</f>
+        <v/>
+      </c>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>Fed Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L62" s="28">
+        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1">
+      <c r="B63" s="32" t="inlineStr">
+        <is>
+          <t>State Standard Deduction</t>
+        </is>
+      </c>
+      <c r="C63" s="33">
+        <f>IF(L68="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L71),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L71))</f>
+        <v/>
+      </c>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>LTCG Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L63" s="28">
+        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" hidden="1" outlineLevel="1">
+      <c r="B64" s="32" t="inlineStr">
+        <is>
+          <t>Net Short-Term Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C64" s="33">
+        <f>(C13-C15)</f>
+        <v/>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>Status Row# (NIIT/CapLoss)</t>
+        </is>
+      </c>
+      <c r="L64" s="28">
+        <f>MATCH(L59,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" hidden="1" outlineLevel="1">
+      <c r="B65" s="32" t="inlineStr">
+        <is>
+          <t>Net Long-Term Gain / (Loss), net of carryforward</t>
+        </is>
+      </c>
+      <c r="C65" s="33">
+        <f>(C14-C16-C17)</f>
+        <v/>
+      </c>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>StdDed Row#</t>
+        </is>
+      </c>
+      <c r="L65" s="28">
+        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" hidden="1" outlineLevel="1">
+      <c r="B66" s="32" t="inlineStr">
+        <is>
+          <t>Combined Net Capital Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C66" s="33">
+        <f>(C64+C65)</f>
+        <v/>
+      </c>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>State Name</t>
+        </is>
+      </c>
+      <c r="L66" s="28">
+        <f>C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" hidden="1" outlineLevel="1">
+      <c r="B67" s="32" t="inlineStr">
+        <is>
+          <t>Ordinary-Taxed Capital Gain / (Loss Deduction, capped)</t>
+        </is>
+      </c>
+      <c r="C67" s="33">
+        <f>IF(C66&lt;=0,MAX(C66,-C60),IF(AND(C64&gt;=0,C65&gt;=0),C64,IF(AND(C64&lt;0,C65&gt;=0),0,IF(AND(C64&gt;=0,C65&lt;0),C66,0))))</f>
+        <v/>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>State Code</t>
+        </is>
+      </c>
+      <c r="L67" s="28">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L66,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" hidden="1" outlineLevel="1">
+      <c r="B68" s="32" t="inlineStr">
+        <is>
+          <t>Preferential (LTCG-Rate) Net Capital Gain</t>
+        </is>
+      </c>
+      <c r="C68" s="33">
+        <f>IF(C66&lt;=0,0,IF(AND(C64&gt;=0,C65&gt;=0),C65,IF(AND(C64&lt;0,C65&gt;=0),C66,IF(AND(C64&gt;=0,C65&lt;0),0,0))))</f>
+        <v/>
+      </c>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>State Category</t>
+        </is>
+      </c>
+      <c r="L68" s="28">
+        <f>IF(L59="Married Filing Jointly","MFJ","Single")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" hidden="1" outlineLevel="1">
+      <c r="B69" s="32" t="inlineStr">
+        <is>
+          <t>Capital Loss Carryforward to Future Years</t>
+        </is>
+      </c>
+      <c r="C69" s="33">
+        <f>IF(C66&lt;=0,C66-MAX(C66,-C60),0)</f>
+        <v/>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>State Key</t>
+        </is>
+      </c>
+      <c r="L69" s="28">
+        <f>L67&amp;"|"&amp;L68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1">
+      <c r="B70" s="32" t="inlineStr">
+        <is>
+          <t>Ordinary Taxable Income Including Gain</t>
+        </is>
+      </c>
+      <c r="C70" s="33">
+        <f>MAX(0,C9+C67)</f>
+        <v/>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>State Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L70" s="28">
+        <f>MATCH(L69,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" hidden="1" outlineLevel="1">
+      <c r="B71" s="32" t="inlineStr">
+        <is>
+          <t>Federal Tax on Taxable Income Alone (no gain)</t>
+        </is>
+      </c>
+      <c r="C71" s="33">
+        <f>SUMPRODUCT((C9&gt;$M$74:$M$80)*($L$74:$L$80)*(MIN(C9,$N$74:$N$80)-$M$74:$M$80))</f>
+        <v/>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>State Master Row#</t>
+        </is>
+      </c>
+      <c r="L71" s="28">
+        <f>MATCH(L67,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" hidden="1" outlineLevel="1">
+      <c r="B72" s="32" t="inlineStr">
+        <is>
+          <t>Federal Tax on Taxable Income Including Short-Term Gain</t>
+        </is>
+      </c>
+      <c r="C72" s="33">
+        <f>SUMPRODUCT((C70&gt;$M$74:$M$80)*($L$74:$L$80)*(MIN(C70,$N$74:$N$80)-$M$74:$M$80))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" hidden="1" outlineLevel="1">
+      <c r="B73" s="35" t="inlineStr">
+        <is>
+          <t>Federal Tax on Short-Term Gain</t>
+        </is>
+      </c>
+      <c r="C73" s="33">
+        <f>MAX(0,C72-C71)</f>
+        <v/>
+      </c>
+      <c r="K73" s="29" t="inlineStr">
+        <is>
+          <t>Federal Ordinary Brackets</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" hidden="1" outlineLevel="1">
+      <c r="B74" s="35" t="inlineStr">
+        <is>
+          <t>Federal Tax on Long-Term Gain (stacked)</t>
+        </is>
+      </c>
+      <c r="C74" s="33">
+        <f>SUMPRODUCT($L$83:$L$85*(MAX(0,MIN((C70+C68),$N$83:$N$85)-MAX(C70,$M$83:$M$85))))</f>
+        <v/>
+      </c>
+      <c r="L74" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="M74" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="N74" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1">
+      <c r="B75" s="32" t="inlineStr">
+        <is>
+          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
+        </is>
+      </c>
+      <c r="C75" s="33">
+        <f>(C9+C59+C67+C68)</f>
+        <v/>
+      </c>
+      <c r="L75" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="M75" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="N75" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" hidden="1" outlineLevel="1">
+      <c r="B76" s="32" t="inlineStr">
+        <is>
+          <t>Net Investment Income (the modeled capital gain)</t>
+        </is>
+      </c>
+      <c r="C76" s="33">
+        <f>MAX(0,C67+C68)</f>
+        <v/>
+      </c>
+      <c r="L76" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="M76" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="N76" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" hidden="1" outlineLevel="1">
+      <c r="B77" s="35" t="inlineStr">
+        <is>
+          <t>NIIT</t>
+        </is>
+      </c>
+      <c r="C77" s="33">
+        <f>C62*MIN(C76,MAX(0,C75-C61))</f>
+        <v/>
+      </c>
+      <c r="L77" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="M77" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="N77" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" hidden="1" outlineLevel="1">
+      <c r="B78" s="32" t="inlineStr">
+        <is>
+          <t>State Taxable Income (gain taxed as ordinary income)</t>
+        </is>
+      </c>
+      <c r="C78" s="33">
+        <f>MAX(0,C9+C67+C68-C63)</f>
+        <v/>
+      </c>
+      <c r="L78" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="M78" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="N78" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" hidden="1" outlineLevel="1">
+      <c r="B79" s="35" t="inlineStr">
+        <is>
+          <t>State Tax</t>
+        </is>
+      </c>
+      <c r="C79" s="33">
+        <f>IF(L67="OTHER",C8*C78,SUMPRODUCT((C78&gt;$M$88:$M$95)*($L$88:$L$95)*(MIN(C78,$N$88:$N$95)-$M$88:$M$95)))</f>
+        <v/>
+      </c>
+      <c r="L79" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="M79" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="N79" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" hidden="1" outlineLevel="1">
+      <c r="B80" s="21" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
         </is>
       </c>
-      <c r="F5" s="22" t="inlineStr">
-        <is>
-          <t>After-Tax Proceeds</t>
-        </is>
-      </c>
-      <c r="G5" s="22" t="inlineStr">
-        <is>
-          <t>Effective Tax Rate on Gain</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="B6" s="23">
-        <f>E62</f>
-        <v/>
-      </c>
-      <c r="C6" s="23">
-        <f>E63</f>
-        <v/>
-      </c>
-      <c r="D6" s="23">
-        <f>E64</f>
-        <v/>
-      </c>
-      <c r="E6" s="23">
-        <f>E65</f>
-        <v/>
-      </c>
-      <c r="F6" s="23">
-        <f>C90</f>
-        <v/>
-      </c>
-      <c r="G6" s="24">
-        <f>C91</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>This reflects the incremental tax created by the Portfolio Sale Scenario in Section 4. See Section 5 for the full before/after comparison.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>1. PERSONAL INFORMATION</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="26" t="inlineStr">
-        <is>
-          <t>Tax Year</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="n">
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="26" t="inlineStr">
-        <is>
-          <t>Filing Status</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Married Filing Jointly</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="26" t="inlineStr">
-        <is>
-          <t>State of Residence</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>New Jersey</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="27" t="inlineStr">
-        <is>
-          <t>State Tax Rate if 'Other (Manual Entry)' Selected</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="28" t="inlineStr">
-        <is>
-          <t>YOUR STATE</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="29" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="C17" s="30">
-        <f>L116</f>
-        <v/>
-      </c>
-      <c r="D17" s="31" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="29" t="inlineStr">
-        <is>
-          <t>Estimated State Marginal Tax Rate</t>
-        </is>
-      </c>
-      <c r="C18" s="32">
-        <f>C176</f>
-        <v/>
-      </c>
-      <c r="D18" s="31" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>(automatically pulled from the Tax Rates &amp; Assumptions tab; updates once you enter income below)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>2. ORDINARY TAXABLE INCOME</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="34" t="inlineStr">
-        <is>
-          <t>Used only to determine where your capital gains fall within the tax brackets - this is your income BEFORE adding the gains being modeled below.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="26" t="inlineStr">
-        <is>
-          <t>Income Entry Method</t>
-        </is>
-      </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>Option B: Gross Income + Deductions</t>
-        </is>
-      </c>
-      <c r="D23" s="31" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="27" t="inlineStr">
-        <is>
-          <t>Option A - Estimated Taxable Income</t>
-        </is>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="27" t="inlineStr">
-        <is>
-          <t>Option B - W-2 / Salary Income</t>
-        </is>
-      </c>
-      <c r="C25" s="13" t="n">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="27" t="inlineStr">
-        <is>
-          <t>Option B - Other Ordinary Income (business, pension, interest, etc.)</t>
-        </is>
-      </c>
-      <c r="C26" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="27" t="inlineStr">
-        <is>
-          <t>Option B - Pre-Tax Retirement Contributions</t>
-        </is>
-      </c>
-      <c r="C27" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="27" t="inlineStr">
-        <is>
-          <t>Option B - Estimated Deductions (standard or itemized)</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="26" t="inlineStr">
-        <is>
-          <t>Estimated Taxable Ordinary Income</t>
-        </is>
-      </c>
-      <c r="C29" s="35">
-        <f>C112</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>3. CAPITAL GAINS &amp; LOSSES (current year, before the sale scenario below)</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="29" t="inlineStr">
-        <is>
-          <t>Short-Term Capital Gains (held one year or less)</t>
-        </is>
-      </c>
-      <c r="C32" s="13" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="29" t="inlineStr">
-        <is>
-          <t>Long-Term Capital Gains (held more than one year)</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="29" t="inlineStr">
-        <is>
-          <t>Short-Term Capital Losses</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="29" t="inlineStr">
-        <is>
-          <t>Long-Term Capital Losses</t>
-        </is>
-      </c>
-      <c r="C35" s="13" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="29" t="inlineStr">
-        <is>
-          <t>Existing Capital Loss Carryforward</t>
-        </is>
-      </c>
-      <c r="C36" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" s="29" t="inlineStr">
-        <is>
-          <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C37" s="36">
-        <f>(C32-C34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="29" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C38" s="36">
-        <f>(C33-C35-C36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="26" t="inlineStr">
-        <is>
-          <t>Total Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C39" s="35">
-        <f>(C37+C38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>4. PORTFOLIO SALE SCENARIO (optional - model a potential sale)</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="4" t="n"/>
-      <c r="E41" s="4" t="n"/>
-      <c r="F41" s="4" t="n"/>
-      <c r="G41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Investment</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>Current Value</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>Cost Basis</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Holding Period</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Estimated Gain / (Loss)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>XYZ Stock</t>
-        </is>
-      </c>
-      <c r="C43" s="13" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D43" s="13" t="n">
-        <v>100000</v>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>Long-Term</t>
-        </is>
-      </c>
-      <c r="F43" s="36">
-        <f>C43-D43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="12" t="inlineStr"/>
-      <c r="C44" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>Long-Term</t>
-        </is>
-      </c>
-      <c r="F44" s="36">
-        <f>C44-D44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="12" t="inlineStr"/>
-      <c r="C45" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>Long-Term</t>
-        </is>
-      </c>
-      <c r="F45" s="36">
-        <f>C45-D45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="12" t="inlineStr"/>
-      <c r="C46" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>Long-Term</t>
-        </is>
-      </c>
-      <c r="F46" s="36">
-        <f>C46-D46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="12" t="inlineStr"/>
-      <c r="C47" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>Long-Term</t>
-        </is>
-      </c>
-      <c r="F47" s="36">
-        <f>C47-D47</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="12" t="inlineStr"/>
-      <c r="C48" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>Long-Term</t>
-        </is>
-      </c>
-      <c r="F48" s="36">
-        <f>C48-D48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="26" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C49" s="37">
-        <f>SUM(C43:C48)</f>
-        <v/>
-      </c>
-      <c r="F49" s="37">
-        <f>SUM(F43:F48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="33" t="inlineStr">
-        <is>
-          <t>Leave the Investment name blank on any row you don't need. Gain/Loss is calculated automatically as Current Value minus Cost Basis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>5. ESTIMATED TAX</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-      <c r="D52" s="4" t="n"/>
-      <c r="E52" s="4" t="n"/>
-      <c r="F52" s="4" t="n"/>
-      <c r="G52" s="4" t="n"/>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="B53" s="38" t="inlineStr">
-        <is>
-          <t>Net Capital Gain / Loss (including the sale scenario above)</t>
-        </is>
-      </c>
-      <c r="C53" s="39" t="n"/>
-    </row>
-    <row r="54">
-      <c r="B54" s="29" t="inlineStr">
-        <is>
-          <t>Total Capital Gains</t>
-        </is>
-      </c>
-      <c r="C54" s="40">
-        <f>((C32+C117)+(C33+C119))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="29" t="inlineStr">
-        <is>
-          <t>Total Capital Losses</t>
-        </is>
-      </c>
-      <c r="C55" s="40">
-        <f>-((C34+C118)+(C35+C120)+C36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="26" t="inlineStr">
-        <is>
-          <t>Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C56" s="41">
-        <f>C143</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="29" t="inlineStr">
-        <is>
-          <t>Current-Year Capital Loss Deduction</t>
-        </is>
-      </c>
-      <c r="C57" s="40">
-        <f>IF(C143&lt;0,MAX(C143,-C113),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="B58" s="29" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward to Future Years</t>
-        </is>
-      </c>
-      <c r="C58" s="40">
-        <f>-C146</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="B60" s="38" t="inlineStr">
-        <is>
-          <t>Before vs. After the Sale</t>
-        </is>
-      </c>
-      <c r="C60" s="39" t="n"/>
-    </row>
-    <row r="61" ht="28" customHeight="1">
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Without Realizing
-the Gain</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>After Realizing
-the Gain</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
-        <is>
-          <t>Incremental
-(From the Sale)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="29" t="inlineStr">
-        <is>
-          <t>Estimated Federal Tax</t>
-        </is>
-      </c>
-      <c r="C62" s="36">
-        <f>C132</f>
-        <v/>
-      </c>
-      <c r="D62" s="36">
-        <f>C150</f>
-        <v/>
-      </c>
-      <c r="E62" s="36">
-        <f>D62-C62</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="29" t="inlineStr">
-        <is>
-          <t>Estimated State Tax</t>
-        </is>
-      </c>
-      <c r="C63" s="36">
-        <f>C137</f>
-        <v/>
-      </c>
-      <c r="D63" s="36">
-        <f>C155</f>
-        <v/>
-      </c>
-      <c r="E63" s="36">
-        <f>D63-C63</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="29" t="inlineStr">
-        <is>
-          <t>Estimated NIIT</t>
-        </is>
-      </c>
-      <c r="C64" s="36">
-        <f>C135</f>
-        <v/>
-      </c>
-      <c r="D64" s="36">
-        <f>C153</f>
-        <v/>
-      </c>
-      <c r="E64" s="36">
-        <f>D64-C64</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="26" t="inlineStr">
-        <is>
-          <t>Total Estimated Tax</t>
-        </is>
-      </c>
-      <c r="C65" s="35">
-        <f>C138</f>
-        <v/>
-      </c>
-      <c r="D65" s="35">
-        <f>C156</f>
-        <v/>
-      </c>
-      <c r="E65" s="35">
-        <f>D65-C65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="B67" s="29" t="inlineStr">
-        <is>
-          <t>Your Long-Term Capital Gains Rate (marginal, after the sale)</t>
-        </is>
-      </c>
-      <c r="C67" s="32">
-        <f>C157</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>Tax Component</t>
-        </is>
-      </c>
-      <c r="G69" s="7" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="F70" s="42" t="inlineStr">
-        <is>
-          <t>Federal Tax</t>
-        </is>
-      </c>
-      <c r="G70" s="43">
-        <f>E62</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="F71" s="42" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="G71" s="43">
-        <f>E63</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="F72" s="42" t="inlineStr">
-        <is>
-          <t>NIIT</t>
-        </is>
-      </c>
-      <c r="G72" s="43">
-        <f>E64</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="3" t="inlineStr">
-        <is>
-          <t>6. AFTER-TAX PROCEEDS (from the Portfolio Sale Scenario)</t>
-        </is>
-      </c>
-      <c r="B87" s="4" t="n"/>
-      <c r="C87" s="4" t="n"/>
-      <c r="D87" s="4" t="n"/>
-      <c r="E87" s="4" t="n"/>
-      <c r="F87" s="4" t="n"/>
-      <c r="G87" s="4" t="n"/>
-    </row>
-    <row r="88">
-      <c r="B88" s="29" t="inlineStr">
-        <is>
-          <t>Sale Proceeds</t>
-        </is>
-      </c>
-      <c r="C88" s="35">
-        <f>C49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="29" t="inlineStr">
-        <is>
-          <t>Less: Estimated Tax From Sale</t>
-        </is>
-      </c>
-      <c r="C89" s="36">
-        <f>-E65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="26" t="inlineStr">
-        <is>
-          <t>Estimated After-Tax Proceeds</t>
-        </is>
-      </c>
-      <c r="C90" s="35">
-        <f>C88+C89</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="29" t="inlineStr">
-        <is>
-          <t>Estimated Tax Rate on Gain</t>
-        </is>
-      </c>
-      <c r="C91" s="44">
-        <f>IFERROR(E65/F49,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="3" t="inlineStr">
-        <is>
-          <t>7. TAX-LOSS HARVESTING - WHAT IF?</t>
-        </is>
-      </c>
-      <c r="B93" s="4" t="n"/>
-      <c r="C93" s="4" t="n"/>
-      <c r="D93" s="4" t="n"/>
-      <c r="E93" s="4" t="n"/>
-      <c r="F93" s="4" t="n"/>
-      <c r="G93" s="4" t="n"/>
-    </row>
-    <row r="94">
-      <c r="B94" s="25" t="inlineStr">
-        <is>
-          <t>Model harvesting an additional loss on top of the sale scenario above (assumed long-term).</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="B95" s="26" t="inlineStr">
-        <is>
-          <t>Potential Additional Loss to Harvest</t>
-        </is>
-      </c>
-      <c r="C95" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="96">
-      <c r="B96" s="29" t="inlineStr">
-        <is>
-          <t>Current Estimated Tax (with sale, before harvesting)</t>
-        </is>
-      </c>
-      <c r="C96" s="36">
-        <f>C156</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97">
-      <c r="B97" s="29" t="inlineStr">
-        <is>
-          <t>Estimated Tax After Harvesting</t>
-        </is>
-      </c>
-      <c r="C97" s="36">
-        <f>C174</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="B98" s="26" t="inlineStr">
-        <is>
-          <t>Estimated Tax Savings From Harvesting</t>
-        </is>
-      </c>
-      <c r="C98" s="35">
-        <f>C96-C97</f>
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="B99" s="29" t="inlineStr">
-        <is>
-          <t>Remaining Capital Loss Carryforward After Harvesting</t>
-        </is>
-      </c>
-      <c r="C99" s="36">
-        <f>-C164</f>
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="B101" s="45" t="inlineStr">
-        <is>
-          <t>Full calculation detail is available below for your advisor. Click the [+] in the row-number margin to expand.</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="B103" s="46" t="inlineStr">
-        <is>
-          <t>Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="107" hidden="1" outlineLevel="1" collapsed="1">
-      <c r="A107" s="47" t="inlineStr">
-        <is>
-          <t>CALCULATION DETAIL (grouped - click + to expand)</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" hidden="1" outlineLevel="1"/>
-    <row r="109" hidden="1" outlineLevel="1">
-      <c r="B109" s="48" t="inlineStr">
-        <is>
-          <t>Standard Deduction (add-back for MAGI estimate)</t>
-        </is>
-      </c>
-      <c r="C109" s="49">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L114)</f>
-        <v/>
-      </c>
-      <c r="K109" s="7" t="inlineStr">
-        <is>
-          <t>Filing Status</t>
-        </is>
-      </c>
-      <c r="L109" s="42">
-        <f>C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="110" hidden="1" outlineLevel="1">
-      <c r="B110" s="48" t="inlineStr">
-        <is>
-          <t>Taxable Ordinary Income - Option A (direct entry)</t>
-        </is>
-      </c>
-      <c r="C110" s="49">
-        <f>C24</f>
-        <v/>
-      </c>
-      <c r="K110" s="7" t="inlineStr">
-        <is>
-          <t>Tax Year</t>
-        </is>
-      </c>
-      <c r="L110" s="42">
-        <f>C11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="111" hidden="1" outlineLevel="1">
-      <c r="B111" s="48" t="inlineStr">
-        <is>
-          <t>Taxable Ordinary Income - Option B (Gross - Pretax - Deductions)</t>
-        </is>
-      </c>
-      <c r="C111" s="49">
-        <f>MAX(0,C25+C26-C27-C28)</f>
-        <v/>
-      </c>
-      <c r="K111" s="7" t="inlineStr">
-        <is>
-          <t>Federal Key</t>
-        </is>
-      </c>
-      <c r="L111" s="42">
-        <f>L110&amp;"|"&amp;L109</f>
-        <v/>
-      </c>
-    </row>
-    <row r="112" hidden="1" outlineLevel="1">
-      <c r="B112" s="50" t="inlineStr">
-        <is>
-          <t>Estimated Taxable Ordinary Income (per method selected)</t>
-        </is>
-      </c>
-      <c r="C112" s="49">
-        <f>IF(C23="Option A: Enter Taxable Income Directly",C110,C111)</f>
-        <v/>
-      </c>
-      <c r="K112" s="7" t="inlineStr">
-        <is>
-          <t>Fed Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L112" s="42">
-        <f>MATCH(L111,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="113" hidden="1" outlineLevel="1">
-      <c r="B113" s="48" t="inlineStr">
-        <is>
-          <t>Capital Loss Limit vs. Ordinary Income</t>
-        </is>
-      </c>
-      <c r="C113" s="49">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L115)</f>
-        <v/>
-      </c>
-      <c r="K113" s="7" t="inlineStr">
-        <is>
-          <t>LTCG Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L113" s="42">
-        <f>MATCH(L111,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="114" hidden="1" outlineLevel="1">
-      <c r="B114" s="48" t="inlineStr">
-        <is>
-          <t>NIIT Threshold</t>
-        </is>
-      </c>
-      <c r="C114" s="49">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L115)</f>
-        <v/>
-      </c>
-      <c r="K114" s="7" t="inlineStr">
-        <is>
-          <t>StdDed Row#</t>
-        </is>
-      </c>
-      <c r="L114" s="42">
-        <f>MATCH(L111,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="115" hidden="1" outlineLevel="1">
-      <c r="B115" s="48" t="inlineStr">
-        <is>
-          <t>NIIT Rate</t>
-        </is>
-      </c>
-      <c r="C115" s="51">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L115)</f>
-        <v/>
-      </c>
-      <c r="K115" s="7" t="inlineStr">
-        <is>
-          <t>Status Row# (NIIT/CapLoss)</t>
-        </is>
-      </c>
-      <c r="L115" s="42">
-        <f>MATCH(L109,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="116" hidden="1" outlineLevel="1">
-      <c r="B116" s="48" t="inlineStr">
-        <is>
-          <t>State Standard Deduction</t>
-        </is>
-      </c>
-      <c r="C116" s="49">
-        <f>IF(L118="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L121),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L121))</f>
-        <v/>
-      </c>
-      <c r="K116" s="7" t="inlineStr">
-        <is>
-          <t>State Name</t>
-        </is>
-      </c>
-      <c r="L116" s="42">
-        <f>C13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="117" hidden="1" outlineLevel="1">
-      <c r="B117" s="48" t="inlineStr">
-        <is>
-          <t>Sale Scenario - Short-Term Gain Total</t>
-        </is>
-      </c>
-      <c r="C117" s="49">
-        <f>SUMIFS(F43:F48,E43:E48,"Short-Term",F43:F48,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="K117" s="7" t="inlineStr">
-        <is>
-          <t>State Code</t>
-        </is>
-      </c>
-      <c r="L117" s="42">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L116,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="118" hidden="1" outlineLevel="1">
-      <c r="B118" s="48" t="inlineStr">
-        <is>
-          <t>Sale Scenario - Short-Term Loss Total</t>
-        </is>
-      </c>
-      <c r="C118" s="49">
-        <f>-SUMIFS(F43:F48,E43:E48,"Short-Term",F43:F48,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="K118" s="7" t="inlineStr">
-        <is>
-          <t>State Category</t>
-        </is>
-      </c>
-      <c r="L118" s="42">
-        <f>IF(L109="Married Filing Jointly","MFJ","Single")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="119" hidden="1" outlineLevel="1">
-      <c r="B119" s="48" t="inlineStr">
-        <is>
-          <t>Sale Scenario - Long-Term Gain Total</t>
-        </is>
-      </c>
-      <c r="C119" s="49">
-        <f>SUMIFS(F43:F48,E43:E48,"Long-Term",F43:F48,"&gt;0")</f>
-        <v/>
-      </c>
-      <c r="K119" s="7" t="inlineStr">
-        <is>
-          <t>State Key</t>
-        </is>
-      </c>
-      <c r="L119" s="42">
-        <f>L117&amp;"|"&amp;L118</f>
-        <v/>
-      </c>
-    </row>
-    <row r="120" hidden="1" outlineLevel="1">
-      <c r="B120" s="48" t="inlineStr">
-        <is>
-          <t>Sale Scenario - Long-Term Loss Total</t>
-        </is>
-      </c>
-      <c r="C120" s="49">
-        <f>-SUMIFS(F43:F48,E43:E48,"Long-Term",F43:F48,"&lt;0")</f>
-        <v/>
-      </c>
-      <c r="K120" s="7" t="inlineStr">
-        <is>
-          <t>State Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L120" s="42">
-        <f>MATCH(L119,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="121" hidden="1" outlineLevel="1">
-      <c r="K121" s="7" t="inlineStr">
-        <is>
-          <t>State Master Row#</t>
-        </is>
-      </c>
-      <c r="L121" s="42">
-        <f>MATCH(L117,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="122" hidden="1" outlineLevel="1">
-      <c r="A122" s="52" t="inlineStr">
-        <is>
-          <t>-- BEFORE (current year only) --</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" hidden="1" outlineLevel="1">
-      <c r="B123" s="53" t="inlineStr">
-        <is>
-          <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C123" s="54">
-        <f>(C32-C34)</f>
-        <v/>
-      </c>
-      <c r="K123" s="52" t="inlineStr">
-        <is>
-          <t>Federal Ordinary Brackets</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" hidden="1" outlineLevel="1">
-      <c r="B124" s="53" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss), net of carryforward</t>
-        </is>
-      </c>
-      <c r="C124" s="54">
-        <f>(C33-C35-C36)</f>
-        <v/>
-      </c>
-      <c r="L124" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="M124" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="N124" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L112)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="125" hidden="1" outlineLevel="1">
-      <c r="B125" s="53" t="inlineStr">
-        <is>
-          <t>Combined Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C125" s="54">
-        <f>(C123+C124)</f>
-        <v/>
-      </c>
-      <c r="L125" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="M125" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="N125" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L112)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="126" hidden="1" outlineLevel="1">
-      <c r="B126" s="53" t="inlineStr">
-        <is>
-          <t>Ordinary-Taxed Capital Gain / (Loss Deduction, capped)</t>
-        </is>
-      </c>
-      <c r="C126" s="54">
-        <f>IF(C125&lt;=0,MAX(C125,-C113),IF(AND(C123&gt;=0,C124&gt;=0),C123,IF(AND(C123&lt;0,C124&gt;=0),0,IF(AND(C123&gt;=0,C124&lt;0),C125,0))))</f>
-        <v/>
-      </c>
-      <c r="L126" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="M126" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="N126" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L112)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="127" hidden="1" outlineLevel="1">
-      <c r="B127" s="53" t="inlineStr">
-        <is>
-          <t>Preferential (LTCG-Rate) Net Capital Gain</t>
-        </is>
-      </c>
-      <c r="C127" s="54">
-        <f>IF(C125&lt;=0,0,IF(AND(C123&gt;=0,C124&gt;=0),C124,IF(AND(C123&lt;0,C124&gt;=0),C125,IF(AND(C123&gt;=0,C124&lt;0),0,0))))</f>
-        <v/>
-      </c>
-      <c r="L127" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="M127" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="N127" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L112)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="128" hidden="1" outlineLevel="1">
-      <c r="B128" s="53" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward to Future Years</t>
-        </is>
-      </c>
-      <c r="C128" s="54">
-        <f>IF(C125&lt;=0,C125-MAX(C125,-C113),0)</f>
-        <v/>
-      </c>
-      <c r="L128" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="M128" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="N128" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L112)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="129" hidden="1" outlineLevel="1">
-      <c r="B129" s="53" t="inlineStr">
-        <is>
-          <t>Ordinary Taxable Income Including Gain</t>
-        </is>
-      </c>
-      <c r="C129" s="54">
-        <f>MAX(0,C112+C126)</f>
-        <v/>
-      </c>
-      <c r="L129" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="M129" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="N129" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L112)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="130" hidden="1" outlineLevel="1">
-      <c r="B130" s="53" t="inlineStr">
-        <is>
-          <t>Federal Ordinary Tax</t>
-        </is>
-      </c>
-      <c r="C130" s="54">
-        <f>SUMPRODUCT((C129&gt;$M$124:$M$130)*($L$124:$L$130)*(MIN(C129,$N$124:$N$130)-$M$124:$M$130))</f>
-        <v/>
-      </c>
-      <c r="L130" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="M130" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L112)</f>
-        <v/>
-      </c>
-      <c r="N130" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L112)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="131" hidden="1" outlineLevel="1">
-      <c r="B131" s="53" t="inlineStr">
-        <is>
-          <t>Federal Long-Term Capital Gains Tax (stacked)</t>
-        </is>
-      </c>
-      <c r="C131" s="54">
-        <f>SUMPRODUCT($L$133:$L$135*(MAX(0,MIN((C129+C127),$N$133:$N$135)-MAX(C129,$M$133:$M$135))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="132" hidden="1" outlineLevel="1">
-      <c r="B132" s="57" t="inlineStr">
-        <is>
-          <t>Total Federal Tax</t>
-        </is>
-      </c>
-      <c r="C132" s="54">
-        <f>(C130+C131)</f>
-        <v/>
-      </c>
-      <c r="K132" s="52" t="inlineStr">
+      <c r="C80" s="36">
+        <f>(C73+C74+C77+C79)</f>
+        <v/>
+      </c>
+      <c r="L80" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="M80" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L62)</f>
+        <v/>
+      </c>
+      <c r="N80" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" hidden="1" outlineLevel="1">
+      <c r="B81" s="32" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate on the Gain</t>
+        </is>
+      </c>
+      <c r="C81" s="37">
+        <f>IFERROR(C80/MAX(0.0001,C66),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" hidden="1" outlineLevel="1">
+      <c r="B82" s="32" t="inlineStr">
+        <is>
+          <t>Marginal LTCG Rate Applied</t>
+        </is>
+      </c>
+      <c r="C82" s="37">
+        <f>IFERROR(INDEX($L$83:$L$85,MATCH(C70,$M$83:$M$85,1)),0)</f>
+        <v/>
+      </c>
+      <c r="K82" s="29" t="inlineStr">
         <is>
           <t>LTCG Brackets</t>
         </is>
       </c>
     </row>
-    <row r="133" hidden="1" outlineLevel="1">
-      <c r="B133" s="53" t="inlineStr">
-        <is>
-          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
-        </is>
-      </c>
-      <c r="C133" s="54">
-        <f>(C112+C109+C126+C127)</f>
-        <v/>
-      </c>
-      <c r="L133" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L113)</f>
-        <v/>
-      </c>
-      <c r="M133" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L113)</f>
-        <v/>
-      </c>
-      <c r="N133" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L113)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="134" hidden="1" outlineLevel="1">
-      <c r="B134" s="53" t="inlineStr">
-        <is>
-          <t>Net Investment Income (the modeled capital gain)</t>
-        </is>
-      </c>
-      <c r="C134" s="54">
-        <f>MAX(0,C126+C127)</f>
-        <v/>
-      </c>
-      <c r="L134" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L113)</f>
-        <v/>
-      </c>
-      <c r="M134" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L113)</f>
-        <v/>
-      </c>
-      <c r="N134" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L113)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="135" hidden="1" outlineLevel="1">
-      <c r="B135" s="57" t="inlineStr">
-        <is>
-          <t>NIIT</t>
-        </is>
-      </c>
-      <c r="C135" s="54">
-        <f>C115*MIN(C134,MAX(0,C133-C114))</f>
-        <v/>
-      </c>
-      <c r="L135" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L113)</f>
-        <v/>
-      </c>
-      <c r="M135" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L113)</f>
-        <v/>
-      </c>
-      <c r="N135" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L113)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="136" hidden="1" outlineLevel="1">
-      <c r="B136" s="53" t="inlineStr">
-        <is>
-          <t>State Taxable Income (gain taxed as ordinary income)</t>
-        </is>
-      </c>
-      <c r="C136" s="54">
-        <f>MAX(0,C112+C126+C127-C116)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="137" hidden="1" outlineLevel="1">
-      <c r="B137" s="57" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="C137" s="54">
-        <f>IF(L117="OTHER",C14*C136,SUMPRODUCT((C136&gt;$M$138:$M$145)*($L$138:$L$145)*(MIN(C136,$N$138:$N$145)-$M$138:$M$145)))</f>
-        <v/>
-      </c>
-      <c r="K137" s="52" t="inlineStr">
+    <row r="83" hidden="1" outlineLevel="1">
+      <c r="L83" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L63)</f>
+        <v/>
+      </c>
+      <c r="M83" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L63)</f>
+        <v/>
+      </c>
+      <c r="N83" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" hidden="1" outlineLevel="1">
+      <c r="L84" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L63)</f>
+        <v/>
+      </c>
+      <c r="M84" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L63)</f>
+        <v/>
+      </c>
+      <c r="N84" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" hidden="1" outlineLevel="1">
+      <c r="L85" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L63)</f>
+        <v/>
+      </c>
+      <c r="M85" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L63)</f>
+        <v/>
+      </c>
+      <c r="N85" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" hidden="1" outlineLevel="1"/>
+    <row r="87" hidden="1" outlineLevel="1">
+      <c r="K87" s="29" t="inlineStr">
         <is>
           <t>State Brackets</t>
         </is>
       </c>
     </row>
-    <row r="138" hidden="1" outlineLevel="1">
-      <c r="B138" s="58" t="inlineStr">
-        <is>
-          <t>Total Estimated Tax (Federal + State + NIIT)</t>
-        </is>
-      </c>
-      <c r="C138" s="59">
-        <f>(C132+C137+C135)</f>
-        <v/>
-      </c>
-      <c r="L138" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M138" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N138" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="139" hidden="1" outlineLevel="1">
-      <c r="B139" s="53" t="inlineStr">
-        <is>
-          <t>Marginal LTCG Rate Applied</t>
-        </is>
-      </c>
-      <c r="C139" s="60">
-        <f>IFERROR(INDEX($L$133:$L$135,MATCH(C129,$M$133:$M$135,1)),0)</f>
-        <v/>
-      </c>
-      <c r="L139" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M139" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N139" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="140" hidden="1" outlineLevel="1">
-      <c r="A140" s="52" t="inlineStr">
-        <is>
-          <t>-- AFTER (current year + sale scenario) --</t>
-        </is>
-      </c>
-      <c r="L140" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M140" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N140" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="141" hidden="1" outlineLevel="1">
-      <c r="B141" s="53" t="inlineStr">
-        <is>
-          <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C141" s="54">
-        <f>((C32+C117)-(C34+C118))</f>
-        <v/>
-      </c>
-      <c r="L141" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M141" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N141" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="142" hidden="1" outlineLevel="1">
-      <c r="B142" s="53" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss), net of carryforward</t>
-        </is>
-      </c>
-      <c r="C142" s="54">
-        <f>((C33+C119)-(C35+C120)-C36)</f>
-        <v/>
-      </c>
-      <c r="L142" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M142" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N142" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="143" hidden="1" outlineLevel="1">
-      <c r="B143" s="53" t="inlineStr">
-        <is>
-          <t>Combined Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C143" s="54">
-        <f>(C141+C142)</f>
-        <v/>
-      </c>
-      <c r="L143" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M143" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N143" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="144" hidden="1" outlineLevel="1">
-      <c r="B144" s="53" t="inlineStr">
-        <is>
-          <t>Ordinary-Taxed Capital Gain / (Loss Deduction, capped)</t>
-        </is>
-      </c>
-      <c r="C144" s="54">
-        <f>IF(C143&lt;=0,MAX(C143,-C113),IF(AND(C141&gt;=0,C142&gt;=0),C141,IF(AND(C141&lt;0,C142&gt;=0),0,IF(AND(C141&gt;=0,C142&lt;0),C143,0))))</f>
-        <v/>
-      </c>
-      <c r="L144" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M144" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N144" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="145" hidden="1" outlineLevel="1">
-      <c r="B145" s="53" t="inlineStr">
-        <is>
-          <t>Preferential (LTCG-Rate) Net Capital Gain</t>
-        </is>
-      </c>
-      <c r="C145" s="54">
-        <f>IF(C143&lt;=0,0,IF(AND(C141&gt;=0,C142&gt;=0),C142,IF(AND(C141&lt;0,C142&gt;=0),C143,IF(AND(C141&gt;=0,C142&lt;0),0,0))))</f>
-        <v/>
-      </c>
-      <c r="L145" s="55">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="M145" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L120)</f>
-        <v/>
-      </c>
-      <c r="N145" s="56">
-        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L120)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="146" hidden="1" outlineLevel="1">
-      <c r="B146" s="53" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward to Future Years</t>
-        </is>
-      </c>
-      <c r="C146" s="54">
-        <f>IF(C143&lt;=0,C143-MAX(C143,-C113),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="147" hidden="1" outlineLevel="1">
-      <c r="B147" s="53" t="inlineStr">
-        <is>
-          <t>Ordinary Taxable Income Including Gain</t>
-        </is>
-      </c>
-      <c r="C147" s="54">
-        <f>MAX(0,C112+C144)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="148" hidden="1" outlineLevel="1">
-      <c r="B148" s="53" t="inlineStr">
-        <is>
-          <t>Federal Ordinary Tax</t>
-        </is>
-      </c>
-      <c r="C148" s="54">
-        <f>SUMPRODUCT((C147&gt;$M$124:$M$130)*($L$124:$L$130)*(MIN(C147,$N$124:$N$130)-$M$124:$M$130))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="149" hidden="1" outlineLevel="1">
-      <c r="B149" s="53" t="inlineStr">
-        <is>
-          <t>Federal Long-Term Capital Gains Tax (stacked)</t>
-        </is>
-      </c>
-      <c r="C149" s="54">
-        <f>SUMPRODUCT($L$133:$L$135*(MAX(0,MIN((C147+C145),$N$133:$N$135)-MAX(C147,$M$133:$M$135))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="150" hidden="1" outlineLevel="1">
-      <c r="B150" s="57" t="inlineStr">
-        <is>
-          <t>Total Federal Tax</t>
-        </is>
-      </c>
-      <c r="C150" s="54">
-        <f>(C148+C149)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="151" hidden="1" outlineLevel="1">
-      <c r="B151" s="53" t="inlineStr">
-        <is>
-          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
-        </is>
-      </c>
-      <c r="C151" s="54">
-        <f>(C112+C109+C144+C145)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="152" hidden="1" outlineLevel="1">
-      <c r="B152" s="53" t="inlineStr">
-        <is>
-          <t>Net Investment Income (the modeled capital gain)</t>
-        </is>
-      </c>
-      <c r="C152" s="54">
-        <f>MAX(0,C144+C145)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="153" hidden="1" outlineLevel="1">
-      <c r="B153" s="57" t="inlineStr">
-        <is>
-          <t>NIIT</t>
-        </is>
-      </c>
-      <c r="C153" s="54">
-        <f>C115*MIN(C152,MAX(0,C151-C114))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="154" hidden="1" outlineLevel="1">
-      <c r="B154" s="53" t="inlineStr">
-        <is>
-          <t>State Taxable Income (gain taxed as ordinary income)</t>
-        </is>
-      </c>
-      <c r="C154" s="54">
-        <f>MAX(0,C112+C144+C145-C116)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="155" hidden="1" outlineLevel="1">
-      <c r="B155" s="57" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="C155" s="54">
-        <f>IF(L117="OTHER",C14*C154,SUMPRODUCT((C154&gt;$M$138:$M$145)*($L$138:$L$145)*(MIN(C154,$N$138:$N$145)-$M$138:$M$145)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156" hidden="1" outlineLevel="1">
-      <c r="B156" s="58" t="inlineStr">
-        <is>
-          <t>Total Estimated Tax (Federal + State + NIIT)</t>
-        </is>
-      </c>
-      <c r="C156" s="59">
-        <f>(C150+C155+C153)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157" hidden="1" outlineLevel="1">
-      <c r="B157" s="53" t="inlineStr">
-        <is>
-          <t>Marginal LTCG Rate Applied</t>
-        </is>
-      </c>
-      <c r="C157" s="60">
-        <f>IFERROR(INDEX($L$133:$L$135,MATCH(C147,$M$133:$M$135,1)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="158" hidden="1" outlineLevel="1">
-      <c r="A158" s="52" t="inlineStr">
-        <is>
-          <t>-- AFTER SALE + TAX-LOSS HARVESTING --</t>
-        </is>
-      </c>
-    </row>
-    <row r="159" hidden="1" outlineLevel="1">
-      <c r="B159" s="53" t="inlineStr">
-        <is>
-          <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C159" s="54">
-        <f>((C32+C117)-(C34+C118))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="160" hidden="1" outlineLevel="1">
-      <c r="B160" s="53" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss), net of carryforward</t>
-        </is>
-      </c>
-      <c r="C160" s="54">
-        <f>((C33+C119)-(C35+C120+C95)-C36)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="161" hidden="1" outlineLevel="1">
-      <c r="B161" s="53" t="inlineStr">
-        <is>
-          <t>Combined Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C161" s="54">
-        <f>(C159+C160)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="162" hidden="1" outlineLevel="1">
-      <c r="B162" s="53" t="inlineStr">
-        <is>
-          <t>Ordinary-Taxed Capital Gain / (Loss Deduction, capped)</t>
-        </is>
-      </c>
-      <c r="C162" s="54">
-        <f>IF(C161&lt;=0,MAX(C161,-C113),IF(AND(C159&gt;=0,C160&gt;=0),C159,IF(AND(C159&lt;0,C160&gt;=0),0,IF(AND(C159&gt;=0,C160&lt;0),C161,0))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="163" hidden="1" outlineLevel="1">
-      <c r="B163" s="53" t="inlineStr">
-        <is>
-          <t>Preferential (LTCG-Rate) Net Capital Gain</t>
-        </is>
-      </c>
-      <c r="C163" s="54">
-        <f>IF(C161&lt;=0,0,IF(AND(C159&gt;=0,C160&gt;=0),C160,IF(AND(C159&lt;0,C160&gt;=0),C161,IF(AND(C159&gt;=0,C160&lt;0),0,0))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="164" hidden="1" outlineLevel="1">
-      <c r="B164" s="53" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward to Future Years</t>
-        </is>
-      </c>
-      <c r="C164" s="54">
-        <f>IF(C161&lt;=0,C161-MAX(C161,-C113),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="165" hidden="1" outlineLevel="1">
-      <c r="B165" s="53" t="inlineStr">
-        <is>
-          <t>Ordinary Taxable Income Including Gain</t>
-        </is>
-      </c>
-      <c r="C165" s="54">
-        <f>MAX(0,C112+C162)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="166" hidden="1" outlineLevel="1">
-      <c r="B166" s="53" t="inlineStr">
-        <is>
-          <t>Federal Ordinary Tax</t>
-        </is>
-      </c>
-      <c r="C166" s="54">
-        <f>SUMPRODUCT((C165&gt;$M$124:$M$130)*($L$124:$L$130)*(MIN(C165,$N$124:$N$130)-$M$124:$M$130))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="167" hidden="1" outlineLevel="1">
-      <c r="B167" s="53" t="inlineStr">
-        <is>
-          <t>Federal Long-Term Capital Gains Tax (stacked)</t>
-        </is>
-      </c>
-      <c r="C167" s="54">
-        <f>SUMPRODUCT($L$133:$L$135*(MAX(0,MIN((C165+C163),$N$133:$N$135)-MAX(C165,$M$133:$M$135))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="168" hidden="1" outlineLevel="1">
-      <c r="B168" s="57" t="inlineStr">
-        <is>
-          <t>Total Federal Tax</t>
-        </is>
-      </c>
-      <c r="C168" s="54">
-        <f>(C166+C167)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="169" hidden="1" outlineLevel="1">
-      <c r="B169" s="53" t="inlineStr">
-        <is>
-          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
-        </is>
-      </c>
-      <c r="C169" s="54">
-        <f>(C112+C109+C162+C163)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="170" hidden="1" outlineLevel="1">
-      <c r="B170" s="53" t="inlineStr">
-        <is>
-          <t>Net Investment Income (the modeled capital gain)</t>
-        </is>
-      </c>
-      <c r="C170" s="54">
-        <f>MAX(0,C162+C163)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="171" hidden="1" outlineLevel="1">
-      <c r="B171" s="57" t="inlineStr">
-        <is>
-          <t>NIIT</t>
-        </is>
-      </c>
-      <c r="C171" s="54">
-        <f>C115*MIN(C170,MAX(0,C169-C114))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="172" hidden="1" outlineLevel="1">
-      <c r="B172" s="53" t="inlineStr">
-        <is>
-          <t>State Taxable Income (gain taxed as ordinary income)</t>
-        </is>
-      </c>
-      <c r="C172" s="54">
-        <f>MAX(0,C112+C162+C163-C116)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="173" hidden="1" outlineLevel="1">
-      <c r="B173" s="57" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="C173" s="54">
-        <f>IF(L117="OTHER",C14*C172,SUMPRODUCT((C172&gt;$M$138:$M$145)*($L$138:$L$145)*(MIN(C172,$N$138:$N$145)-$M$138:$M$145)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="174" hidden="1" outlineLevel="1">
-      <c r="B174" s="58" t="inlineStr">
-        <is>
-          <t>Total Estimated Tax (Federal + State + NIIT)</t>
-        </is>
-      </c>
-      <c r="C174" s="59">
-        <f>(C168+C173+C171)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="175" hidden="1" outlineLevel="1">
-      <c r="B175" s="53" t="inlineStr">
-        <is>
-          <t>Marginal LTCG Rate Applied</t>
-        </is>
-      </c>
-      <c r="C175" s="60">
-        <f>IFERROR(INDEX($L$133:$L$135,MATCH(C165,$M$133:$M$135,1)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="176" hidden="1" outlineLevel="1">
-      <c r="B176" s="53" t="inlineStr">
-        <is>
-          <t>State Marginal Tax Rate (on ordinary income, before any gain)</t>
-        </is>
-      </c>
-      <c r="C176" s="60">
-        <f>IF(L117="OTHER",C14,IFERROR(INDEX($L$138:$L$145,MATCH(MAX(0,C112-C116),$M$138:$M$145,1)),0))</f>
-        <v/>
-      </c>
-    </row>
+    <row r="88" hidden="1" outlineLevel="1">
+      <c r="L88" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M88" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N88" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" hidden="1" outlineLevel="1">
+      <c r="L89" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M89" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N89" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" hidden="1" outlineLevel="1">
+      <c r="L90" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M90" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N90" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" hidden="1" outlineLevel="1">
+      <c r="L91" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M91" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N91" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" hidden="1" outlineLevel="1">
+      <c r="L92" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M92" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N92" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" hidden="1" outlineLevel="1">
+      <c r="L93" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M93" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N93" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" hidden="1" outlineLevel="1">
+      <c r="L94" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M94" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N94" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" hidden="1" outlineLevel="1">
+      <c r="L95" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="M95" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L70)</f>
+        <v/>
+      </c>
+      <c r="N95" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L70)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" hidden="1" outlineLevel="1"/>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="A52:G52"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A93:G93"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B103:G105"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B101:F101"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B94:G94"/>
-    <mergeCell ref="A87:G87"/>
-    <mergeCell ref="B50:G50"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="C18:D18"/>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="B53:F55"/>
   </mergeCells>
-  <dataValidations count="10">
-    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2024,2025"</formula1>
     </dataValidation>
-    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Single,Married Filing Jointly,Married Filing Separately,Head of Household"</formula1>
     </dataValidation>
-    <dataValidation sqref="C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>='Tax Rates &amp; Assumptions'!$B$46:$B$77</formula1>
-    </dataValidation>
-    <dataValidation sqref="C23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Option A: Enter Taxable Income Directly,Option B: Gross Income + Deductions"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Short-Term,Long-Term"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Short-Term,Long-Term"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Short-Term,Long-Term"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Short-Term,Long-Term"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Short-Term,Long-Term"</formula1>
-    </dataValidation>
-    <dataValidation sqref="E48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Short-Term,Long-Term"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix misleading state tax rate display
The only rate-looking field near State of Residence was the manual
override input (default 5%, meant to apply only when State = Other),
so it looked like every state showed a flat 5% regardless of selection
-- the underlying state tax calculation was already state-specific and
correct. Added back a real auto-computed "Estimated State Marginal Tax
Rate" that looks up the selected state's actual bracket via the state
bracket table and the entered taxable income, and relabeled the manual
override to make its conditional purpose explicit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XveA8LngnD1MFNqnzekQW3
</commit_message>
<xml_diff>
--- a/Capital_Gains_Tax_Estimator.xlsx
+++ b/Capital_Gains_Tax_Estimator.xlsx
@@ -104,14 +104,20 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -164,12 +170,6 @@
       <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="16"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -236,7 +236,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -283,24 +283,27 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -310,28 +313,28 @@
     <xf numFmtId="10" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="24" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="25" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="25" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -437,7 +440,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Capital Gains Tax Calculator'!G36</f>
+              <f>'Capital Gains Tax Calculator'!G38</f>
             </strRef>
           </tx>
           <spPr>
@@ -447,12 +450,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Capital Gains Tax Calculator'!$F$37:$F$39</f>
+              <f>'Capital Gains Tax Calculator'!$F$39:$F$41</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Capital Gains Tax Calculator'!$G$37:$G$39</f>
+              <f>'Capital Gains Tax Calculator'!$G$39:$G$41</f>
             </numRef>
           </val>
         </ser>
@@ -477,7 +480,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>35</row>
+      <row>37</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2700000"/>
@@ -787,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N95"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -866,172 +869,168 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="22" t="inlineStr">
-        <is>
-          <t>State Tax Rate if 'Other (Manual Entry)' Selected</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="n">
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Estimated State Marginal Tax Rate</t>
+        </is>
+      </c>
+      <c r="C8" s="22">
+        <f>C85</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>(automatically pulled from the Tax Rates &amp; Assumptions tab based on your state and taxable income below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Manual State Tax Rate Override - used ONLY if State of Residence = 'Other (Manual Entry)'</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="21" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Taxable Income (before these gains/losses)</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C11" s="13" t="n">
         <v>200000</v>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="23" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>(your salary/other income after deductions - used only to determine which tax brackets your gains fall into)</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>CAPITAL GAINS &amp; LOSSES</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="25" t="inlineStr">
         <is>
           <t>Short-Term Capital Gains (held 1 year or less)</t>
         </is>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C15" s="13" t="n">
         <v>3000</v>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="24" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="25" t="inlineStr">
         <is>
           <t>Long-Term Capital Gains (held more than 1 year)</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C16" s="13" t="n">
         <v>155000</v>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="24" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="25" t="inlineStr">
         <is>
           <t>Short-Term Capital Losses</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="24" t="inlineStr">
+      <c r="C17" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>Long-Term Capital Losses</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C18" s="13" t="n">
         <v>2000</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="24" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="25" t="inlineStr">
         <is>
           <t>Capital Loss Carryforward (from prior years)</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="C19" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>ESTIMATED TAX</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="B20" s="25" t="inlineStr">
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="B22" s="26" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
         </is>
       </c>
-      <c r="C20" s="25" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>Effective Tax Rate</t>
         </is>
       </c>
-      <c r="D20" s="25" t="inlineStr">
+      <c r="D22" s="26" t="inlineStr">
         <is>
           <t>Federal Tax</t>
         </is>
       </c>
-      <c r="E20" s="25" t="inlineStr">
+      <c r="E22" s="26" t="inlineStr">
         <is>
           <t>State Tax</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="B21" s="38">
-        <f>C80</f>
-        <v/>
-      </c>
-      <c r="C21" s="39">
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="39">
+        <f>C82</f>
+        <v/>
+      </c>
+      <c r="C23" s="40">
+        <f>C83</f>
+        <v/>
+      </c>
+      <c r="D23" s="39">
+        <f>(C75+C76)</f>
+        <v/>
+      </c>
+      <c r="E23" s="39">
         <f>C81</f>
         <v/>
       </c>
-      <c r="D21" s="38">
-        <f>(C73+C74)</f>
-        <v/>
-      </c>
-      <c r="E21" s="38">
-        <f>C79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="24" t="inlineStr">
+    </row>
+    <row r="25">
+      <c r="B25" s="25" t="inlineStr">
         <is>
           <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C23" s="40">
-        <f>C64</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="24" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C24" s="40">
-        <f>C65</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Total Net Capital Gain / (Loss)</t>
         </is>
       </c>
       <c r="C25" s="41">
@@ -1040,97 +1039,97 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="25" t="inlineStr">
+        <is>
+          <t>Net Long-Term Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C26" s="41">
+        <f>C67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>Total Net Capital Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C27" s="42">
+        <f>C68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>Capital Loss Deduction (against ordinary income)</t>
         </is>
       </c>
-      <c r="C26" s="40">
-        <f>IF(C66&lt;0,MAX(C66,-C60),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="24" t="inlineStr">
+      <c r="C28" s="41">
+        <f>IF(C68&lt;0,MAX(C68,-C62),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="25" t="inlineStr">
         <is>
           <t>Capital Loss Carryforward to Future Years</t>
         </is>
       </c>
-      <c r="C27" s="40">
-        <f>-C69</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="24" t="inlineStr">
+      <c r="C29" s="41">
+        <f>-C71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="25" t="inlineStr">
         <is>
           <t>Federal Tax on Short-Term Gain (ordinary rates)</t>
         </is>
       </c>
-      <c r="C28" s="40">
-        <f>C73</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="24" t="inlineStr">
+      <c r="C30" s="41">
+        <f>C75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="25" t="inlineStr">
         <is>
           <t>Federal Tax on Long-Term Gain (preferential rates)</t>
         </is>
       </c>
-      <c r="C29" s="40">
-        <f>C74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="24" t="inlineStr">
+      <c r="C31" s="41">
+        <f>C76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="25" t="inlineStr">
         <is>
           <t>Net Investment Income Tax (NIIT)</t>
         </is>
       </c>
-      <c r="C30" s="40">
-        <f>C77</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="24" t="inlineStr">
+      <c r="C32" s="41">
+        <f>C79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>State Tax</t>
         </is>
       </c>
-      <c r="C31" s="40">
-        <f>C79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="21" t="inlineStr">
+      <c r="C33" s="41">
+        <f>C81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
-        </is>
-      </c>
-      <c r="C32" s="41">
-        <f>C80</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="24" t="inlineStr">
-        <is>
-          <t>Effective Tax Rate on the Gain</t>
-        </is>
-      </c>
-      <c r="C33" s="42">
-        <f>C81</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="24" t="inlineStr">
-        <is>
-          <t>Marginal Long-Term Capital Gains Rate</t>
         </is>
       </c>
       <c r="C34" s="42">
@@ -1138,715 +1137,747 @@
         <v/>
       </c>
     </row>
+    <row r="35">
+      <c r="B35" s="25" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate on the Gain</t>
+        </is>
+      </c>
+      <c r="C35" s="43">
+        <f>C83</f>
+        <v/>
+      </c>
+    </row>
     <row r="36">
-      <c r="F36" s="7" t="inlineStr">
+      <c r="B36" s="25" t="inlineStr">
+        <is>
+          <t>Marginal Long-Term Capital Gains Rate</t>
+        </is>
+      </c>
+      <c r="C36" s="43">
+        <f>C84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="F38" s="7" t="inlineStr">
         <is>
           <t>Tax Component</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G38" s="7" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="F37" s="28" t="inlineStr">
+    <row r="39">
+      <c r="F39" s="29" t="inlineStr">
         <is>
           <t>Federal Tax</t>
         </is>
       </c>
-      <c r="G37" s="43">
-        <f>(C73+C74)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="F38" s="28" t="inlineStr">
+      <c r="G39" s="44">
+        <f>(C75+C76)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="F40" s="29" t="inlineStr">
         <is>
           <t>State Tax</t>
         </is>
       </c>
-      <c r="G38" s="43">
+      <c r="G40" s="44">
+        <f>C81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="F41" s="29" t="inlineStr">
+        <is>
+          <t>NIIT</t>
+        </is>
+      </c>
+      <c r="G41" s="44">
         <f>C79</f>
         <v/>
       </c>
     </row>
-    <row r="39">
-      <c r="F39" s="28" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="27" t="inlineStr">
+        <is>
+          <t>Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="59" hidden="1" outlineLevel="1" collapsed="1">
+      <c r="A59" s="28" t="inlineStr">
+        <is>
+          <t>CALCULATION DETAIL (grouped - click + to expand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" hidden="1" outlineLevel="1"/>
+    <row r="61" hidden="1" outlineLevel="1">
+      <c r="B61" s="33" t="inlineStr">
+        <is>
+          <t>Standard Deduction (add-back for MAGI estimate)</t>
+        </is>
+      </c>
+      <c r="C61" s="34">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L67)</f>
+        <v/>
+      </c>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t>Filing Status</t>
+        </is>
+      </c>
+      <c r="L61" s="29">
+        <f>C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" hidden="1" outlineLevel="1">
+      <c r="B62" s="33" t="inlineStr">
+        <is>
+          <t>Capital Loss Limit vs. Ordinary Income</t>
+        </is>
+      </c>
+      <c r="C62" s="34">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L66)</f>
+        <v/>
+      </c>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>Tax Year</t>
+        </is>
+      </c>
+      <c r="L62" s="29">
+        <f>C5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1">
+      <c r="B63" s="33" t="inlineStr">
+        <is>
+          <t>NIIT Threshold</t>
+        </is>
+      </c>
+      <c r="C63" s="34">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L66)</f>
+        <v/>
+      </c>
+      <c r="K63" s="7" t="inlineStr">
+        <is>
+          <t>Federal Key</t>
+        </is>
+      </c>
+      <c r="L63" s="29">
+        <f>L62&amp;"|"&amp;L61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" hidden="1" outlineLevel="1">
+      <c r="B64" s="33" t="inlineStr">
+        <is>
+          <t>NIIT Rate</t>
+        </is>
+      </c>
+      <c r="C64" s="35">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L66)</f>
+        <v/>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>Fed Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L64" s="29">
+        <f>MATCH(L63,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" hidden="1" outlineLevel="1">
+      <c r="B65" s="33" t="inlineStr">
+        <is>
+          <t>State Standard Deduction</t>
+        </is>
+      </c>
+      <c r="C65" s="34">
+        <f>IF(L70="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L73),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L73))</f>
+        <v/>
+      </c>
+      <c r="K65" s="7" t="inlineStr">
+        <is>
+          <t>LTCG Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L65" s="29">
+        <f>MATCH(L63,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" hidden="1" outlineLevel="1">
+      <c r="B66" s="33" t="inlineStr">
+        <is>
+          <t>Net Short-Term Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C66" s="34">
+        <f>(C15-C17)</f>
+        <v/>
+      </c>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>Status Row# (NIIT/CapLoss)</t>
+        </is>
+      </c>
+      <c r="L66" s="29">
+        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" hidden="1" outlineLevel="1">
+      <c r="B67" s="33" t="inlineStr">
+        <is>
+          <t>Net Long-Term Gain / (Loss), net of carryforward</t>
+        </is>
+      </c>
+      <c r="C67" s="34">
+        <f>(C16-C18-C19)</f>
+        <v/>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>StdDed Row#</t>
+        </is>
+      </c>
+      <c r="L67" s="29">
+        <f>MATCH(L63,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" hidden="1" outlineLevel="1">
+      <c r="B68" s="33" t="inlineStr">
+        <is>
+          <t>Combined Net Capital Gain / (Loss)</t>
+        </is>
+      </c>
+      <c r="C68" s="34">
+        <f>(C66+C67)</f>
+        <v/>
+      </c>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>State Name</t>
+        </is>
+      </c>
+      <c r="L68" s="29">
+        <f>C7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" hidden="1" outlineLevel="1">
+      <c r="B69" s="33" t="inlineStr">
+        <is>
+          <t>Ordinary-Taxed Capital Gain / (Loss Deduction, capped)</t>
+        </is>
+      </c>
+      <c r="C69" s="34">
+        <f>IF(C68&lt;=0,MAX(C68,-C62),IF(AND(C66&gt;=0,C67&gt;=0),C66,IF(AND(C66&lt;0,C67&gt;=0),0,IF(AND(C66&gt;=0,C67&lt;0),C68,0))))</f>
+        <v/>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>State Code</t>
+        </is>
+      </c>
+      <c r="L69" s="29">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L68,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1">
+      <c r="B70" s="33" t="inlineStr">
+        <is>
+          <t>Preferential (LTCG-Rate) Net Capital Gain</t>
+        </is>
+      </c>
+      <c r="C70" s="34">
+        <f>IF(C68&lt;=0,0,IF(AND(C66&gt;=0,C67&gt;=0),C67,IF(AND(C66&lt;0,C67&gt;=0),C68,IF(AND(C66&gt;=0,C67&lt;0),0,0))))</f>
+        <v/>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>State Category</t>
+        </is>
+      </c>
+      <c r="L70" s="29">
+        <f>IF(L61="Married Filing Jointly","MFJ","Single")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" hidden="1" outlineLevel="1">
+      <c r="B71" s="33" t="inlineStr">
+        <is>
+          <t>Capital Loss Carryforward to Future Years</t>
+        </is>
+      </c>
+      <c r="C71" s="34">
+        <f>IF(C68&lt;=0,C68-MAX(C68,-C62),0)</f>
+        <v/>
+      </c>
+      <c r="K71" s="7" t="inlineStr">
+        <is>
+          <t>State Key</t>
+        </is>
+      </c>
+      <c r="L71" s="29">
+        <f>L69&amp;"|"&amp;L70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" hidden="1" outlineLevel="1">
+      <c r="B72" s="33" t="inlineStr">
+        <is>
+          <t>Ordinary Taxable Income Including Gain</t>
+        </is>
+      </c>
+      <c r="C72" s="34">
+        <f>MAX(0,C11+C69)</f>
+        <v/>
+      </c>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>State Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L72" s="29">
+        <f>MATCH(L71,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" hidden="1" outlineLevel="1">
+      <c r="B73" s="33" t="inlineStr">
+        <is>
+          <t>Federal Tax on Taxable Income Alone (no gain)</t>
+        </is>
+      </c>
+      <c r="C73" s="34">
+        <f>SUMPRODUCT((C11&gt;$M$76:$M$82)*($L$76:$L$82)*(MIN(C11,$N$76:$N$82)-$M$76:$M$82))</f>
+        <v/>
+      </c>
+      <c r="K73" s="7" t="inlineStr">
+        <is>
+          <t>State Master Row#</t>
+        </is>
+      </c>
+      <c r="L73" s="29">
+        <f>MATCH(L69,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" hidden="1" outlineLevel="1">
+      <c r="B74" s="33" t="inlineStr">
+        <is>
+          <t>Federal Tax on Taxable Income Including Short-Term Gain</t>
+        </is>
+      </c>
+      <c r="C74" s="34">
+        <f>SUMPRODUCT((C72&gt;$M$76:$M$82)*($L$76:$L$82)*(MIN(C72,$N$76:$N$82)-$M$76:$M$82))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1">
+      <c r="B75" s="36" t="inlineStr">
+        <is>
+          <t>Federal Tax on Short-Term Gain</t>
+        </is>
+      </c>
+      <c r="C75" s="34">
+        <f>MAX(0,C74-C73)</f>
+        <v/>
+      </c>
+      <c r="K75" s="30" t="inlineStr">
+        <is>
+          <t>Federal Ordinary Brackets</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" hidden="1" outlineLevel="1">
+      <c r="B76" s="36" t="inlineStr">
+        <is>
+          <t>Federal Tax on Long-Term Gain (stacked)</t>
+        </is>
+      </c>
+      <c r="C76" s="34">
+        <f>SUMPRODUCT($L$85:$L$87*(MAX(0,MIN((C72+C70),$N$85:$N$87)-MAX(C72,$M$85:$M$87))))</f>
+        <v/>
+      </c>
+      <c r="L76" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="M76" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="N76" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" hidden="1" outlineLevel="1">
+      <c r="B77" s="33" t="inlineStr">
+        <is>
+          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
+        </is>
+      </c>
+      <c r="C77" s="34">
+        <f>(C11+C61+C69+C70)</f>
+        <v/>
+      </c>
+      <c r="L77" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="M77" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="N77" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" hidden="1" outlineLevel="1">
+      <c r="B78" s="33" t="inlineStr">
+        <is>
+          <t>Net Investment Income (the modeled capital gain)</t>
+        </is>
+      </c>
+      <c r="C78" s="34">
+        <f>MAX(0,C69+C70)</f>
+        <v/>
+      </c>
+      <c r="L78" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="M78" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="N78" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" hidden="1" outlineLevel="1">
+      <c r="B79" s="36" t="inlineStr">
         <is>
           <t>NIIT</t>
         </is>
       </c>
-      <c r="G39" s="43">
-        <f>C77</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="B53" s="26" t="inlineStr">
-        <is>
-          <t>Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="57" hidden="1" outlineLevel="1" collapsed="1">
-      <c r="A57" s="27" t="inlineStr">
-        <is>
-          <t>CALCULATION DETAIL (grouped - click + to expand)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" hidden="1" outlineLevel="1"/>
-    <row r="59" hidden="1" outlineLevel="1">
-      <c r="B59" s="32" t="inlineStr">
-        <is>
-          <t>Standard Deduction (add-back for MAGI estimate)</t>
-        </is>
-      </c>
-      <c r="C59" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L65)</f>
-        <v/>
-      </c>
-      <c r="K59" s="7" t="inlineStr">
-        <is>
-          <t>Filing Status</t>
-        </is>
-      </c>
-      <c r="L59" s="28">
-        <f>C6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" hidden="1" outlineLevel="1">
-      <c r="B60" s="32" t="inlineStr">
-        <is>
-          <t>Capital Loss Limit vs. Ordinary Income</t>
-        </is>
-      </c>
-      <c r="C60" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L64)</f>
-        <v/>
-      </c>
-      <c r="K60" s="7" t="inlineStr">
-        <is>
-          <t>Tax Year</t>
-        </is>
-      </c>
-      <c r="L60" s="28">
-        <f>C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" hidden="1" outlineLevel="1">
-      <c r="B61" s="32" t="inlineStr">
-        <is>
-          <t>NIIT Threshold</t>
-        </is>
-      </c>
-      <c r="C61" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L64)</f>
-        <v/>
-      </c>
-      <c r="K61" s="7" t="inlineStr">
-        <is>
-          <t>Federal Key</t>
-        </is>
-      </c>
-      <c r="L61" s="28">
-        <f>L60&amp;"|"&amp;L59</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" hidden="1" outlineLevel="1">
-      <c r="B62" s="32" t="inlineStr">
-        <is>
-          <t>NIIT Rate</t>
-        </is>
-      </c>
-      <c r="C62" s="34">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L64)</f>
-        <v/>
-      </c>
-      <c r="K62" s="7" t="inlineStr">
-        <is>
-          <t>Fed Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L62" s="28">
-        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" hidden="1" outlineLevel="1">
-      <c r="B63" s="32" t="inlineStr">
-        <is>
-          <t>State Standard Deduction</t>
-        </is>
-      </c>
-      <c r="C63" s="33">
-        <f>IF(L68="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L71),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L71))</f>
-        <v/>
-      </c>
-      <c r="K63" s="7" t="inlineStr">
-        <is>
-          <t>LTCG Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L63" s="28">
-        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" hidden="1" outlineLevel="1">
-      <c r="B64" s="32" t="inlineStr">
-        <is>
-          <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C64" s="33">
-        <f>(C13-C15)</f>
-        <v/>
-      </c>
-      <c r="K64" s="7" t="inlineStr">
-        <is>
-          <t>Status Row# (NIIT/CapLoss)</t>
-        </is>
-      </c>
-      <c r="L64" s="28">
-        <f>MATCH(L59,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" hidden="1" outlineLevel="1">
-      <c r="B65" s="32" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss), net of carryforward</t>
-        </is>
-      </c>
-      <c r="C65" s="33">
-        <f>(C14-C16-C17)</f>
-        <v/>
-      </c>
-      <c r="K65" s="7" t="inlineStr">
-        <is>
-          <t>StdDed Row#</t>
-        </is>
-      </c>
-      <c r="L65" s="28">
-        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66" hidden="1" outlineLevel="1">
-      <c r="B66" s="32" t="inlineStr">
-        <is>
-          <t>Combined Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C66" s="33">
-        <f>(C64+C65)</f>
-        <v/>
-      </c>
-      <c r="K66" s="7" t="inlineStr">
-        <is>
-          <t>State Name</t>
-        </is>
-      </c>
-      <c r="L66" s="28">
-        <f>C7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" hidden="1" outlineLevel="1">
-      <c r="B67" s="32" t="inlineStr">
-        <is>
-          <t>Ordinary-Taxed Capital Gain / (Loss Deduction, capped)</t>
-        </is>
-      </c>
-      <c r="C67" s="33">
-        <f>IF(C66&lt;=0,MAX(C66,-C60),IF(AND(C64&gt;=0,C65&gt;=0),C64,IF(AND(C64&lt;0,C65&gt;=0),0,IF(AND(C64&gt;=0,C65&lt;0),C66,0))))</f>
-        <v/>
-      </c>
-      <c r="K67" s="7" t="inlineStr">
-        <is>
-          <t>State Code</t>
-        </is>
-      </c>
-      <c r="L67" s="28">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L66,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68" hidden="1" outlineLevel="1">
-      <c r="B68" s="32" t="inlineStr">
-        <is>
-          <t>Preferential (LTCG-Rate) Net Capital Gain</t>
-        </is>
-      </c>
-      <c r="C68" s="33">
-        <f>IF(C66&lt;=0,0,IF(AND(C64&gt;=0,C65&gt;=0),C65,IF(AND(C64&lt;0,C65&gt;=0),C66,IF(AND(C64&gt;=0,C65&lt;0),0,0))))</f>
-        <v/>
-      </c>
-      <c r="K68" s="7" t="inlineStr">
-        <is>
-          <t>State Category</t>
-        </is>
-      </c>
-      <c r="L68" s="28">
-        <f>IF(L59="Married Filing Jointly","MFJ","Single")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" hidden="1" outlineLevel="1">
-      <c r="B69" s="32" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward to Future Years</t>
-        </is>
-      </c>
-      <c r="C69" s="33">
-        <f>IF(C66&lt;=0,C66-MAX(C66,-C60),0)</f>
-        <v/>
-      </c>
-      <c r="K69" s="7" t="inlineStr">
-        <is>
-          <t>State Key</t>
-        </is>
-      </c>
-      <c r="L69" s="28">
-        <f>L67&amp;"|"&amp;L68</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" hidden="1" outlineLevel="1">
-      <c r="B70" s="32" t="inlineStr">
-        <is>
-          <t>Ordinary Taxable Income Including Gain</t>
-        </is>
-      </c>
-      <c r="C70" s="33">
-        <f>MAX(0,C9+C67)</f>
-        <v/>
-      </c>
-      <c r="K70" s="7" t="inlineStr">
-        <is>
-          <t>State Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L70" s="28">
-        <f>MATCH(L69,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" hidden="1" outlineLevel="1">
-      <c r="B71" s="32" t="inlineStr">
-        <is>
-          <t>Federal Tax on Taxable Income Alone (no gain)</t>
-        </is>
-      </c>
-      <c r="C71" s="33">
-        <f>SUMPRODUCT((C9&gt;$M$74:$M$80)*($L$74:$L$80)*(MIN(C9,$N$74:$N$80)-$M$74:$M$80))</f>
-        <v/>
-      </c>
-      <c r="K71" s="7" t="inlineStr">
-        <is>
-          <t>State Master Row#</t>
-        </is>
-      </c>
-      <c r="L71" s="28">
-        <f>MATCH(L67,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" hidden="1" outlineLevel="1">
-      <c r="B72" s="32" t="inlineStr">
-        <is>
-          <t>Federal Tax on Taxable Income Including Short-Term Gain</t>
-        </is>
-      </c>
-      <c r="C72" s="33">
-        <f>SUMPRODUCT((C70&gt;$M$74:$M$80)*($L$74:$L$80)*(MIN(C70,$N$74:$N$80)-$M$74:$M$80))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" hidden="1" outlineLevel="1">
-      <c r="B73" s="35" t="inlineStr">
-        <is>
-          <t>Federal Tax on Short-Term Gain</t>
-        </is>
-      </c>
-      <c r="C73" s="33">
-        <f>MAX(0,C72-C71)</f>
-        <v/>
-      </c>
-      <c r="K73" s="29" t="inlineStr">
-        <is>
-          <t>Federal Ordinary Brackets</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" hidden="1" outlineLevel="1">
-      <c r="B74" s="35" t="inlineStr">
-        <is>
-          <t>Federal Tax on Long-Term Gain (stacked)</t>
-        </is>
-      </c>
-      <c r="C74" s="33">
-        <f>SUMPRODUCT($L$83:$L$85*(MAX(0,MIN((C70+C68),$N$83:$N$85)-MAX(C70,$M$83:$M$85))))</f>
-        <v/>
-      </c>
-      <c r="L74" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="M74" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="N74" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" hidden="1" outlineLevel="1">
-      <c r="B75" s="32" t="inlineStr">
-        <is>
-          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
-        </is>
-      </c>
-      <c r="C75" s="33">
-        <f>(C9+C59+C67+C68)</f>
-        <v/>
-      </c>
-      <c r="L75" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="M75" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="N75" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" hidden="1" outlineLevel="1">
-      <c r="B76" s="32" t="inlineStr">
-        <is>
-          <t>Net Investment Income (the modeled capital gain)</t>
-        </is>
-      </c>
-      <c r="C76" s="33">
-        <f>MAX(0,C67+C68)</f>
-        <v/>
-      </c>
-      <c r="L76" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="M76" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="N76" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" hidden="1" outlineLevel="1">
-      <c r="B77" s="35" t="inlineStr">
-        <is>
-          <t>NIIT</t>
-        </is>
-      </c>
-      <c r="C77" s="33">
-        <f>C62*MIN(C76,MAX(0,C75-C61))</f>
-        <v/>
-      </c>
-      <c r="L77" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="M77" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="N77" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78" hidden="1" outlineLevel="1">
-      <c r="B78" s="32" t="inlineStr">
+      <c r="C79" s="34">
+        <f>C64*MIN(C78,MAX(0,C77-C63))</f>
+        <v/>
+      </c>
+      <c r="L79" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="M79" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="N79" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" hidden="1" outlineLevel="1">
+      <c r="B80" s="33" t="inlineStr">
         <is>
           <t>State Taxable Income (gain taxed as ordinary income)</t>
         </is>
       </c>
-      <c r="C78" s="33">
-        <f>MAX(0,C9+C67+C68-C63)</f>
-        <v/>
-      </c>
-      <c r="L78" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="M78" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="N78" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" hidden="1" outlineLevel="1">
-      <c r="B79" s="35" t="inlineStr">
+      <c r="C80" s="34">
+        <f>MAX(0,C11+C69+C70-C65)</f>
+        <v/>
+      </c>
+      <c r="L80" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="M80" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="N80" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" hidden="1" outlineLevel="1">
+      <c r="B81" s="36" t="inlineStr">
         <is>
           <t>State Tax</t>
         </is>
       </c>
-      <c r="C79" s="33">
-        <f>IF(L67="OTHER",C8*C78,SUMPRODUCT((C78&gt;$M$88:$M$95)*($L$88:$L$95)*(MIN(C78,$N$88:$N$95)-$M$88:$M$95)))</f>
-        <v/>
-      </c>
-      <c r="L79" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="M79" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="N79" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80" hidden="1" outlineLevel="1">
-      <c r="B80" s="21" t="inlineStr">
+      <c r="C81" s="34">
+        <f>IF(L69="OTHER",C10*C80,SUMPRODUCT((C80&gt;$M$90:$M$97)*($L$90:$L$97)*(MIN(C80,$N$90:$N$97)-$M$90:$M$97)))</f>
+        <v/>
+      </c>
+      <c r="L81" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="M81" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="N81" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" hidden="1" outlineLevel="1">
+      <c r="B82" s="21" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
         </is>
       </c>
-      <c r="C80" s="36">
-        <f>(C73+C74+C77+C79)</f>
-        <v/>
-      </c>
-      <c r="L80" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="M80" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L62)</f>
-        <v/>
-      </c>
-      <c r="N80" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" hidden="1" outlineLevel="1">
-      <c r="B81" s="32" t="inlineStr">
+      <c r="C82" s="37">
+        <f>(C75+C76+C79+C81)</f>
+        <v/>
+      </c>
+      <c r="L82" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="M82" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L64)</f>
+        <v/>
+      </c>
+      <c r="N82" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L64)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" hidden="1" outlineLevel="1">
+      <c r="B83" s="33" t="inlineStr">
         <is>
           <t>Effective Tax Rate on the Gain</t>
         </is>
       </c>
-      <c r="C81" s="37">
-        <f>IFERROR(C80/MAX(0.0001,C66),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" hidden="1" outlineLevel="1">
-      <c r="B82" s="32" t="inlineStr">
+      <c r="C83" s="38">
+        <f>IFERROR(C82/MAX(0.0001,C68),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" hidden="1" outlineLevel="1">
+      <c r="B84" s="33" t="inlineStr">
         <is>
           <t>Marginal LTCG Rate Applied</t>
         </is>
       </c>
-      <c r="C82" s="37">
-        <f>IFERROR(INDEX($L$83:$L$85,MATCH(C70,$M$83:$M$85,1)),0)</f>
-        <v/>
-      </c>
-      <c r="K82" s="29" t="inlineStr">
+      <c r="C84" s="38">
+        <f>IFERROR(INDEX($L$85:$L$87,MATCH(C72,$M$85:$M$87,1)),0)</f>
+        <v/>
+      </c>
+      <c r="K84" s="30" t="inlineStr">
         <is>
           <t>LTCG Brackets</t>
         </is>
       </c>
     </row>
-    <row r="83" hidden="1" outlineLevel="1">
-      <c r="L83" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L63)</f>
-        <v/>
-      </c>
-      <c r="M83" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L63)</f>
-        <v/>
-      </c>
-      <c r="N83" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L63)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" hidden="1" outlineLevel="1">
-      <c r="L84" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L63)</f>
-        <v/>
-      </c>
-      <c r="M84" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L63)</f>
-        <v/>
-      </c>
-      <c r="N84" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L63)</f>
-        <v/>
-      </c>
-    </row>
     <row r="85" hidden="1" outlineLevel="1">
-      <c r="L85" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L63)</f>
-        <v/>
-      </c>
-      <c r="M85" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L63)</f>
-        <v/>
-      </c>
-      <c r="N85" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L63)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86" hidden="1" outlineLevel="1"/>
+      <c r="B85" s="33" t="inlineStr">
+        <is>
+          <t>State Marginal Tax Rate (on taxable income before any gain)</t>
+        </is>
+      </c>
+      <c r="C85" s="38">
+        <f>IF(L69="OTHER",C10,IFERROR(INDEX($L$90:$L$97,MATCH(MAX(0,C11-C65),$M$90:$M$97,1)),0))</f>
+        <v/>
+      </c>
+      <c r="L85" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L65)</f>
+        <v/>
+      </c>
+      <c r="M85" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L65)</f>
+        <v/>
+      </c>
+      <c r="N85" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" hidden="1" outlineLevel="1">
+      <c r="L86" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L65)</f>
+        <v/>
+      </c>
+      <c r="M86" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L65)</f>
+        <v/>
+      </c>
+      <c r="N86" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L65)</f>
+        <v/>
+      </c>
+    </row>
     <row r="87" hidden="1" outlineLevel="1">
-      <c r="K87" s="29" t="inlineStr">
+      <c r="L87" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L65)</f>
+        <v/>
+      </c>
+      <c r="M87" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L65)</f>
+        <v/>
+      </c>
+      <c r="N87" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L65)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" hidden="1" outlineLevel="1"/>
+    <row r="89" hidden="1" outlineLevel="1">
+      <c r="K89" s="30" t="inlineStr">
         <is>
           <t>State Brackets</t>
         </is>
       </c>
     </row>
-    <row r="88" hidden="1" outlineLevel="1">
-      <c r="L88" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M88" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N88" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L70)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89" hidden="1" outlineLevel="1">
-      <c r="L89" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M89" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N89" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L70)</f>
-        <v/>
-      </c>
-    </row>
     <row r="90" hidden="1" outlineLevel="1">
-      <c r="L90" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M90" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N90" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L70)</f>
+      <c r="L90" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M90" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N90" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L72)</f>
         <v/>
       </c>
     </row>
     <row r="91" hidden="1" outlineLevel="1">
-      <c r="L91" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M91" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N91" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L70)</f>
+      <c r="L91" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M91" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N91" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L72)</f>
         <v/>
       </c>
     </row>
     <row r="92" hidden="1" outlineLevel="1">
-      <c r="L92" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M92" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N92" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L70)</f>
+      <c r="L92" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M92" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N92" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L72)</f>
         <v/>
       </c>
     </row>
     <row r="93" hidden="1" outlineLevel="1">
-      <c r="L93" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M93" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N93" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L70)</f>
+      <c r="L93" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M93" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N93" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L72)</f>
         <v/>
       </c>
     </row>
     <row r="94" hidden="1" outlineLevel="1">
-      <c r="L94" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M94" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N94" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L70)</f>
+      <c r="L94" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M94" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N94" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L72)</f>
         <v/>
       </c>
     </row>
     <row r="95" hidden="1" outlineLevel="1">
-      <c r="L95" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="M95" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L70)</f>
-        <v/>
-      </c>
-      <c r="N95" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L70)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96" hidden="1" outlineLevel="1"/>
+      <c r="L95" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M95" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N95" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" hidden="1" outlineLevel="1">
+      <c r="L96" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M96" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N96" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" hidden="1" outlineLevel="1">
+      <c r="L97" s="31">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="M97" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L72)</f>
+        <v/>
+      </c>
+      <c r="N97" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" hidden="1" outlineLevel="1"/>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="B55:F57"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A12:F12"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="B53:F55"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="B9:F9"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>

<commit_message>
Rebuild Capital Gains Tax Calculator to match a compact reference UI
Restructured around a single sale (Initial Value / Sale Value / Length
of Ownership) instead of separate gain/loss line items, matching a
simple calculator layout: 3 rows of inputs, a collapsible Advanced
section (401k/IRA/itemized deductions/personal exemptions/locality),
one large "Total Capital Gains Tax You Will Pay" banner, and a
Federal/State/Local/Total table with marginal + effective rate +
amount per row. NIIT is folded into the Federal line. Local tax uses
the existing locality rate table; state personal exemptions use one
generic per-exemption amount (documented on the Tax Rates tab). Same
verified bracket-stacking math as before, re-verified by hand-tracing
the formula chain against a worked example.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XveA8LngnD1MFNqnzekQW3
</commit_message>
<xml_diff>
--- a/Capital_Gains_Tax_Estimator.xlsx
+++ b/Capital_Gains_Tax_Estimator.xlsx
@@ -17,11 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$#,##0;($#,##0)"/>
+    <numFmt numFmtId="166" formatCode="&quot;Total Capital Gains Tax You Will Pay: &quot;$#,##0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="28">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,6 +76,17 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="11"/>
@@ -94,7 +106,7 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00C00000"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -105,31 +117,32 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00595959"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
+      <color rgb="002E5395"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
+      <color rgb="001F3864"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00BF8F00"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00C00000"/>
       <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -169,7 +182,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="001F3864"/>
-      <sz val="16"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -236,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -269,75 +282,69 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="17" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="25" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="27" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -412,93 +419,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Estimated Tax - By Type</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <pieChart>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Capital Gains Tax Calculator'!G38</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Capital Gains Tax Calculator'!$F$39:$F$41</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Capital Gains Tax Calculator'!$G$39:$G$41</f>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showPercent val="1"/>
-        </dLbls>
-        <firstSliceAng val="0"/>
-      </pieChart>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>37</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4320000" cy="2700000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -790,16 +710,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N97"/>
+  <dimension ref="A1:N74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="3" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
@@ -809,176 +732,161 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>CAPITAL GAINS TAX CALCULATOR</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
-        <is>
-          <t>Estimated tax from capital gains and losses. For planning purposes only - not tax, legal, or accounting advice.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>YOUR INFO</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Estimated for planning purposes only - not tax, legal, or accounting advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="23" t="inlineStr">
+        <is>
+          <t>Initial Value</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
+        <is>
+          <t>Sale Value</t>
+        </is>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>Length of Ownership</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="B5" s="21" t="inlineStr">
+      <c r="C5" s="13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>More than a year</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Location (State)</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Annual Income</t>
+        </is>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>Filing Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Married Filing Jointly</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Tax Year</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+    </row>
+    <row r="10">
+      <c r="C10" s="12" t="n">
         <v>2025</v>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Filing Status</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Married Filing Jointly</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>State of Residence</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>New Jersey</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="21" t="inlineStr">
-        <is>
-          <t>Estimated State Marginal Tax Rate</t>
-        </is>
-      </c>
-      <c r="C8" s="22">
-        <f>C85</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>(automatically pulled from the Tax Rates &amp; Assumptions tab based on your state and taxable income below)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>Manual State Tax Rate Override - used ONLY if State of Residence = 'Other (Manual Entry)'</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>Taxable Income (before these gains/losses)</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="n">
-        <v>200000</v>
-      </c>
-    </row>
     <row r="12">
-      <c r="B12" s="23" t="inlineStr">
-        <is>
-          <t>(your salary/other income after deductions - used only to determine which tax brackets your gains fall into)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>CAPITAL GAINS &amp; LOSSES</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="25" t="inlineStr">
-        <is>
-          <t>Short-Term Capital Gains (held 1 year or less)</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="25" t="inlineStr">
-        <is>
-          <t>Long-Term Capital Gains (held more than 1 year)</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>155000</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="25" t="inlineStr">
-        <is>
-          <t>Short-Term Capital Losses</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="25" t="inlineStr">
-        <is>
-          <t>Long-Term Capital Losses</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="25" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward (from prior years)</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>ADVANCED (optional - click the [+] in the row-number margin to expand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" hidden="1" outlineLevel="1" collapsed="1">
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>401(k) Contribution</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>IRA Contribution</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Itemized Deductions</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" hidden="1" outlineLevel="1">
+      <c r="C14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" hidden="1" outlineLevel="1">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Number of Personal Exemptions (state only)</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Locality / City (optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1" outlineLevel="1">
+      <c r="C16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>None / Not Applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="25">
+        <f>C63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1"/>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>ESTIMATED TAX</t>
+          <t>YOUR CAPITAL GAINS TAXES</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -986,912 +894,893 @@
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="B22" s="26" t="inlineStr">
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Tax Type</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Marginal Tax Rate</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Tax Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="D23" s="40">
+        <f>C64</f>
+        <v/>
+      </c>
+      <c r="F23" s="40">
+        <f>C65</f>
+        <v/>
+      </c>
+      <c r="H23" s="41">
+        <f>C56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="23" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D24" s="40">
+        <f>C66</f>
+        <v/>
+      </c>
+      <c r="F24" s="40">
+        <f>C67</f>
+        <v/>
+      </c>
+      <c r="H24" s="41">
+        <f>C61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="D25" s="40">
+        <f>C42</f>
+        <v/>
+      </c>
+      <c r="F25" s="40">
+        <f>C68</f>
+        <v/>
+      </c>
+      <c r="H25" s="41">
+        <f>C62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
         </is>
       </c>
-      <c r="C22" s="26" t="inlineStr">
-        <is>
-          <t>Effective Tax Rate</t>
-        </is>
-      </c>
-      <c r="D22" s="26" t="inlineStr">
-        <is>
-          <t>Federal Tax</t>
-        </is>
-      </c>
-      <c r="E22" s="26" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
-      <c r="B23" s="39">
-        <f>C82</f>
-        <v/>
-      </c>
-      <c r="C23" s="40">
-        <f>C83</f>
-        <v/>
-      </c>
-      <c r="D23" s="39">
-        <f>(C75+C76)</f>
-        <v/>
-      </c>
-      <c r="E23" s="39">
-        <f>C81</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="25" t="inlineStr">
-        <is>
-          <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C25" s="41">
-        <f>C66</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="25" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C26" s="41">
-        <f>C67</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="21" t="inlineStr">
-        <is>
-          <t>Total Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C27" s="42">
-        <f>C68</f>
+      <c r="H26" s="42">
+        <f>C63</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="25" t="inlineStr">
-        <is>
-          <t>Capital Loss Deduction (against ordinary income)</t>
-        </is>
-      </c>
-      <c r="C28" s="41">
-        <f>IF(C68&lt;0,MAX(C68,-C62),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="25" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward to Future Years</t>
-        </is>
-      </c>
-      <c r="C29" s="41">
-        <f>-C71</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="25" t="inlineStr">
-        <is>
-          <t>Federal Tax on Short-Term Gain (ordinary rates)</t>
-        </is>
-      </c>
-      <c r="C30" s="41">
-        <f>C75</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="25" t="inlineStr">
-        <is>
-          <t>Federal Tax on Long-Term Gain (preferential rates)</t>
-        </is>
-      </c>
-      <c r="C31" s="41">
-        <f>C76</f>
-        <v/>
-      </c>
-    </row>
+      <c r="B28" s="27" t="inlineStr">
+        <is>
+          <t>Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions. "Federal" includes the Net Investment Income Tax (3.8%) where applicable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
     <row r="32">
-      <c r="B32" s="25" t="inlineStr">
-        <is>
-          <t>Net Investment Income Tax (NIIT)</t>
-        </is>
-      </c>
-      <c r="C32" s="41">
-        <f>C79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="25" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="C33" s="41">
-        <f>C81</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="21" t="inlineStr">
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>Full calculation detail is available below for your advisor. Click the [+] in the row-number margin to expand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1" collapsed="1">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>CALCULATION DETAIL (grouped - click + to expand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1"/>
+    <row r="36" hidden="1" outlineLevel="1">
+      <c r="B36" s="34" t="inlineStr">
+        <is>
+          <t>Standard Deduction (add-back for MAGI estimate)</t>
+        </is>
+      </c>
+      <c r="C36" s="35">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L42)</f>
+        <v/>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>Filing Status</t>
+        </is>
+      </c>
+      <c r="L36" s="30">
+        <f>I8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1">
+      <c r="B37" s="34" t="inlineStr">
+        <is>
+          <t>Capital Loss Limit vs. Ordinary Income</t>
+        </is>
+      </c>
+      <c r="C37" s="35">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L41)</f>
+        <v/>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>Tax Year</t>
+        </is>
+      </c>
+      <c r="L37" s="30">
+        <f>C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1">
+      <c r="B38" s="34" t="inlineStr">
+        <is>
+          <t>NIIT Threshold</t>
+        </is>
+      </c>
+      <c r="C38" s="35">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L41)</f>
+        <v/>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>Federal Key</t>
+        </is>
+      </c>
+      <c r="L38" s="30">
+        <f>L37&amp;"|"&amp;L36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" hidden="1" outlineLevel="1">
+      <c r="B39" s="34" t="inlineStr">
+        <is>
+          <t>NIIT Rate</t>
+        </is>
+      </c>
+      <c r="C39" s="36">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L41)</f>
+        <v/>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>Fed Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L39" s="30">
+        <f>MATCH(L38,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1">
+      <c r="B40" s="34" t="inlineStr">
+        <is>
+          <t>State Standard Deduction</t>
+        </is>
+      </c>
+      <c r="C40" s="35">
+        <f>IF(L45="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L48),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L48))</f>
+        <v/>
+      </c>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t>LTCG Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L40" s="30">
+        <f>MATCH(L38,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1">
+      <c r="B41" s="34" t="inlineStr">
+        <is>
+          <t>Personal Exemption Amount (per exemption, state)</t>
+        </is>
+      </c>
+      <c r="C41" s="35">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$C$164:$C$164,1)</f>
+        <v/>
+      </c>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t>Status Row# (NIIT/CapLoss)</t>
+        </is>
+      </c>
+      <c r="L41" s="30">
+        <f>MATCH(L36,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1">
+      <c r="B42" s="34" t="inlineStr">
+        <is>
+          <t>Local Tax Rate</t>
+        </is>
+      </c>
+      <c r="C42" s="36">
+        <f>IF(L50=0,0,INDEX('Tax Rates &amp; Assumptions'!$D$148:$D$161,L50))</f>
+        <v/>
+      </c>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t>StdDed Row#</t>
+        </is>
+      </c>
+      <c r="L42" s="30">
+        <f>MATCH(L38,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" hidden="1" outlineLevel="1">
+      <c r="B43" s="34" t="inlineStr">
+        <is>
+          <t>Capital Gain / (Loss) on Sale</t>
+        </is>
+      </c>
+      <c r="C43" s="35">
+        <f>(F5-C5)</f>
+        <v/>
+      </c>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t>State Name</t>
+        </is>
+      </c>
+      <c r="L43" s="30">
+        <f>C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" hidden="1" outlineLevel="1">
+      <c r="B44" s="34" t="inlineStr">
+        <is>
+          <t>Is Long-Term?</t>
+        </is>
+      </c>
+      <c r="C44" s="35">
+        <f>IF(I5="More than a year",1,0)</f>
+        <v/>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>State Code</t>
+        </is>
+      </c>
+      <c r="L44" s="30">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L43,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" hidden="1" outlineLevel="1">
+      <c r="B45" s="34" t="inlineStr">
+        <is>
+          <t>Ordinary-Taxed Portion (short-term gain, or loss deduction capped)</t>
+        </is>
+      </c>
+      <c r="C45" s="35">
+        <f>IF(C43&gt;=0,IF(C44=1,0,C43),MAX(C43,-C37))</f>
+        <v/>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>State Category</t>
+        </is>
+      </c>
+      <c r="L45" s="30">
+        <f>IF(L36="Married Filing Jointly","MFJ","Single")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1">
+      <c r="B46" s="34" t="inlineStr">
+        <is>
+          <t>Preferential-Rate Portion (long-term gain)</t>
+        </is>
+      </c>
+      <c r="C46" s="35">
+        <f>IF(C43&gt;=0,IF(C44=1,C43,0),0)</f>
+        <v/>
+      </c>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t>State Key</t>
+        </is>
+      </c>
+      <c r="L46" s="30">
+        <f>L44&amp;"|"&amp;L45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" hidden="1" outlineLevel="1">
+      <c r="B47" s="34" t="inlineStr">
+        <is>
+          <t>Taxable Income Before the Gain</t>
+        </is>
+      </c>
+      <c r="C47" s="35">
+        <f>MAX(0,F8-C14-F14-MAX(I14,INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L42)))</f>
+        <v/>
+      </c>
+      <c r="K47" s="7" t="inlineStr">
+        <is>
+          <t>State Bracket Row#</t>
+        </is>
+      </c>
+      <c r="L47" s="30">
+        <f>MATCH(L46,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" hidden="1" outlineLevel="1">
+      <c r="B48" s="34" t="inlineStr">
+        <is>
+          <t>Taxable Income Including the Gain</t>
+        </is>
+      </c>
+      <c r="C48" s="35">
+        <f>MAX(0,C47+C45)</f>
+        <v/>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>State Master Row#</t>
+        </is>
+      </c>
+      <c r="L48" s="30">
+        <f>MATCH(L44,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" hidden="1" outlineLevel="1">
+      <c r="B49" s="34" t="inlineStr">
+        <is>
+          <t>Federal Tax on Income Alone (no gain)</t>
+        </is>
+      </c>
+      <c r="C49" s="35">
+        <f>SUMPRODUCT((C47&gt;$M$53:$M$59)*($L$53:$L$59)*(MIN(C47,$N$53:$N$59)-$M$53:$M$59))</f>
+        <v/>
+      </c>
+      <c r="K49" s="7" t="inlineStr">
+        <is>
+          <t>Locality Name</t>
+        </is>
+      </c>
+      <c r="L49" s="30">
+        <f>F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1">
+      <c r="B50" s="34" t="inlineStr">
+        <is>
+          <t>Federal Tax on Income Including the Gain</t>
+        </is>
+      </c>
+      <c r="C50" s="35">
+        <f>SUMPRODUCT((C48&gt;$M$53:$M$59)*($L$53:$L$59)*(MIN(C48,$N$53:$N$59)-$M$53:$M$59))</f>
+        <v/>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>Locality Row#</t>
+        </is>
+      </c>
+      <c r="L50" s="30">
+        <f>IFERROR(MATCH(L49,'Tax Rates &amp; Assumptions'!$B$148:$B$161,0),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" hidden="1" outlineLevel="1">
+      <c r="B51" s="34" t="inlineStr">
+        <is>
+          <t>Federal Tax on Ordinary Portion of the Gain</t>
+        </is>
+      </c>
+      <c r="C51" s="35">
+        <f>C50-C49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" hidden="1" outlineLevel="1">
+      <c r="B52" s="34" t="inlineStr">
+        <is>
+          <t>Federal Tax on Preferential (Long-Term) Portion (stacked)</t>
+        </is>
+      </c>
+      <c r="C52" s="35">
+        <f>SUMPRODUCT($L$62:$L$64*(MAX(0,MIN((C48+C46),$N$62:$N$64)-MAX(C48,$M$62:$M$64))))</f>
+        <v/>
+      </c>
+      <c r="K52" s="31" t="inlineStr">
+        <is>
+          <t>Federal Ordinary Brackets</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" hidden="1" outlineLevel="1">
+      <c r="B53" s="34" t="inlineStr">
+        <is>
+          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
+        </is>
+      </c>
+      <c r="C53" s="35">
+        <f>(C47+C36+C45+C46)</f>
+        <v/>
+      </c>
+      <c r="L53" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="M53" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="N53" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" hidden="1" outlineLevel="1">
+      <c r="B54" s="34" t="inlineStr">
+        <is>
+          <t>Net Investment Income (the modeled gain)</t>
+        </is>
+      </c>
+      <c r="C54" s="35">
+        <f>MAX(0,C45+C46)</f>
+        <v/>
+      </c>
+      <c r="L54" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="M54" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="N54" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" hidden="1" outlineLevel="1">
+      <c r="B55" s="34" t="inlineStr">
+        <is>
+          <t>NIIT</t>
+        </is>
+      </c>
+      <c r="C55" s="35">
+        <f>C39*MIN(C54,MAX(0,C53-C38))</f>
+        <v/>
+      </c>
+      <c r="L55" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="M55" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="N55" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" hidden="1" outlineLevel="1">
+      <c r="B56" s="37" t="inlineStr">
+        <is>
+          <t>Total Federal Tax From the Gain (incl. NIIT)</t>
+        </is>
+      </c>
+      <c r="C56" s="35">
+        <f>(C51+C52+C55)</f>
+        <v/>
+      </c>
+      <c r="L56" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="M56" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="N56" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" hidden="1" outlineLevel="1">
+      <c r="B57" s="34" t="inlineStr">
+        <is>
+          <t>State Taxable Income Before the Gain</t>
+        </is>
+      </c>
+      <c r="C57" s="35">
+        <f>MAX(0,C47-C40-C16*C41)</f>
+        <v/>
+      </c>
+      <c r="L57" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="M57" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="N57" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" hidden="1" outlineLevel="1">
+      <c r="B58" s="34" t="inlineStr">
+        <is>
+          <t>State Taxable Income Including the Gain</t>
+        </is>
+      </c>
+      <c r="C58" s="35">
+        <f>MAX(0,C47+C45+C46-C40-C16*C41)</f>
+        <v/>
+      </c>
+      <c r="L58" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="M58" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="N58" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" hidden="1" outlineLevel="1">
+      <c r="B59" s="34" t="inlineStr">
+        <is>
+          <t>State Tax on Income Alone</t>
+        </is>
+      </c>
+      <c r="C59" s="35">
+        <f>IF(L44="OTHER",0,SUMPRODUCT((C57&gt;$M$67:$M$74)*($L$67:$L$74)*(MIN(C57,$N$67:$N$74)-$M$67:$M$74)))</f>
+        <v/>
+      </c>
+      <c r="L59" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="M59" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L39)</f>
+        <v/>
+      </c>
+      <c r="N59" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" hidden="1" outlineLevel="1">
+      <c r="B60" s="34" t="inlineStr">
+        <is>
+          <t>State Tax on Income Including the Gain</t>
+        </is>
+      </c>
+      <c r="C60" s="35">
+        <f>IF(L44="OTHER",0,SUMPRODUCT((C58&gt;$M$67:$M$74)*($L$67:$L$74)*(MIN(C58,$N$67:$N$74)-$M$67:$M$74)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" hidden="1" outlineLevel="1">
+      <c r="B61" s="37" t="inlineStr">
+        <is>
+          <t>State Tax From the Gain</t>
+        </is>
+      </c>
+      <c r="C61" s="35">
+        <f>(C60-C59)</f>
+        <v/>
+      </c>
+      <c r="K61" s="31" t="inlineStr">
+        <is>
+          <t>LTCG Brackets</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" hidden="1" outlineLevel="1">
+      <c r="B62" s="37" t="inlineStr">
+        <is>
+          <t>Local Tax From the Gain</t>
+        </is>
+      </c>
+      <c r="C62" s="35">
+        <f>C42*MAX(0,C43)</f>
+        <v/>
+      </c>
+      <c r="L62" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L40)</f>
+        <v/>
+      </c>
+      <c r="M62" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L40)</f>
+        <v/>
+      </c>
+      <c r="N62" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1">
+      <c r="B63" s="23" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
         </is>
       </c>
-      <c r="C34" s="42">
-        <f>C82</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="25" t="inlineStr">
-        <is>
-          <t>Effective Tax Rate on the Gain</t>
-        </is>
-      </c>
-      <c r="C35" s="43">
-        <f>C83</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="25" t="inlineStr">
-        <is>
-          <t>Marginal Long-Term Capital Gains Rate</t>
-        </is>
-      </c>
-      <c r="C36" s="43">
-        <f>C84</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>Tax Component</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="F39" s="29" t="inlineStr">
-        <is>
-          <t>Federal Tax</t>
-        </is>
-      </c>
-      <c r="G39" s="44">
-        <f>(C75+C76)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="F40" s="29" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="G40" s="44">
-        <f>C81</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="F41" s="29" t="inlineStr">
-        <is>
-          <t>NIIT</t>
-        </is>
-      </c>
-      <c r="G41" s="44">
-        <f>C79</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" s="27" t="inlineStr">
-        <is>
-          <t>Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="59" hidden="1" outlineLevel="1" collapsed="1">
-      <c r="A59" s="28" t="inlineStr">
-        <is>
-          <t>CALCULATION DETAIL (grouped - click + to expand)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" hidden="1" outlineLevel="1"/>
-    <row r="61" hidden="1" outlineLevel="1">
-      <c r="B61" s="33" t="inlineStr">
-        <is>
-          <t>Standard Deduction (add-back for MAGI estimate)</t>
-        </is>
-      </c>
-      <c r="C61" s="34">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L67)</f>
-        <v/>
-      </c>
-      <c r="K61" s="7" t="inlineStr">
-        <is>
-          <t>Filing Status</t>
-        </is>
-      </c>
-      <c r="L61" s="29">
-        <f>C6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62" hidden="1" outlineLevel="1">
-      <c r="B62" s="33" t="inlineStr">
-        <is>
-          <t>Capital Loss Limit vs. Ordinary Income</t>
-        </is>
-      </c>
-      <c r="C62" s="34">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L66)</f>
-        <v/>
-      </c>
-      <c r="K62" s="7" t="inlineStr">
-        <is>
-          <t>Tax Year</t>
-        </is>
-      </c>
-      <c r="L62" s="29">
-        <f>C5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" hidden="1" outlineLevel="1">
-      <c r="B63" s="33" t="inlineStr">
-        <is>
-          <t>NIIT Threshold</t>
-        </is>
-      </c>
-      <c r="C63" s="34">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L66)</f>
-        <v/>
-      </c>
-      <c r="K63" s="7" t="inlineStr">
-        <is>
-          <t>Federal Key</t>
-        </is>
-      </c>
-      <c r="L63" s="29">
-        <f>L62&amp;"|"&amp;L61</f>
+      <c r="C63" s="38">
+        <f>(C56+C61+C62)</f>
+        <v/>
+      </c>
+      <c r="L63" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L40)</f>
+        <v/>
+      </c>
+      <c r="M63" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L40)</f>
+        <v/>
+      </c>
+      <c r="N63" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L40)</f>
         <v/>
       </c>
     </row>
     <row r="64" hidden="1" outlineLevel="1">
-      <c r="B64" s="33" t="inlineStr">
-        <is>
-          <t>NIIT Rate</t>
-        </is>
-      </c>
-      <c r="C64" s="35">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L66)</f>
-        <v/>
-      </c>
-      <c r="K64" s="7" t="inlineStr">
-        <is>
-          <t>Fed Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L64" s="29">
-        <f>MATCH(L63,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
+      <c r="B64" s="34" t="inlineStr">
+        <is>
+          <t>Federal Marginal Rate Applied to the Gain</t>
+        </is>
+      </c>
+      <c r="C64" s="39">
+        <f>IF(AND(C43&gt;=0,C44=1),IFERROR(INDEX($L$62:$L$64,MATCH(C48,$M$62:$M$64,1)),0),IFERROR(INDEX($L$53:$L$59,MATCH(C48,$M$53:$M$59,1)),0))</f>
+        <v/>
+      </c>
+      <c r="L64" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L40)</f>
+        <v/>
+      </c>
+      <c r="M64" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L40)</f>
+        <v/>
+      </c>
+      <c r="N64" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L40)</f>
         <v/>
       </c>
     </row>
     <row r="65" hidden="1" outlineLevel="1">
-      <c r="B65" s="33" t="inlineStr">
-        <is>
-          <t>State Standard Deduction</t>
-        </is>
-      </c>
-      <c r="C65" s="34">
-        <f>IF(L70="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L73),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L73))</f>
-        <v/>
-      </c>
-      <c r="K65" s="7" t="inlineStr">
-        <is>
-          <t>LTCG Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L65" s="29">
-        <f>MATCH(L63,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
+      <c r="B65" s="34" t="inlineStr">
+        <is>
+          <t>Federal Effective Rate on the Gain</t>
+        </is>
+      </c>
+      <c r="C65" s="39">
+        <f>IFERROR(C56/C43,0)</f>
         <v/>
       </c>
     </row>
     <row r="66" hidden="1" outlineLevel="1">
-      <c r="B66" s="33" t="inlineStr">
-        <is>
-          <t>Net Short-Term Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C66" s="34">
-        <f>(C15-C17)</f>
-        <v/>
-      </c>
-      <c r="K66" s="7" t="inlineStr">
-        <is>
-          <t>Status Row# (NIIT/CapLoss)</t>
-        </is>
-      </c>
-      <c r="L66" s="29">
-        <f>MATCH(L61,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
-        <v/>
+      <c r="B66" s="34" t="inlineStr">
+        <is>
+          <t>State Marginal Rate Applied to the Gain</t>
+        </is>
+      </c>
+      <c r="C66" s="39">
+        <f>IF(L44="OTHER",0,IFERROR(INDEX($L$67:$L$74,MATCH(C58,$M$67:$M$74,1)),0))</f>
+        <v/>
+      </c>
+      <c r="K66" s="31" t="inlineStr">
+        <is>
+          <t>State Brackets</t>
+        </is>
       </c>
     </row>
     <row r="67" hidden="1" outlineLevel="1">
-      <c r="B67" s="33" t="inlineStr">
-        <is>
-          <t>Net Long-Term Gain / (Loss), net of carryforward</t>
-        </is>
-      </c>
-      <c r="C67" s="34">
-        <f>(C16-C18-C19)</f>
-        <v/>
-      </c>
-      <c r="K67" s="7" t="inlineStr">
-        <is>
-          <t>StdDed Row#</t>
-        </is>
-      </c>
-      <c r="L67" s="29">
-        <f>MATCH(L63,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
+      <c r="B67" s="34" t="inlineStr">
+        <is>
+          <t>State Effective Rate on the Gain</t>
+        </is>
+      </c>
+      <c r="C67" s="39">
+        <f>IFERROR(C61/C43,0)</f>
+        <v/>
+      </c>
+      <c r="L67" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M67" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N67" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L47)</f>
         <v/>
       </c>
     </row>
     <row r="68" hidden="1" outlineLevel="1">
-      <c r="B68" s="33" t="inlineStr">
-        <is>
-          <t>Combined Net Capital Gain / (Loss)</t>
-        </is>
-      </c>
-      <c r="C68" s="34">
-        <f>(C66+C67)</f>
-        <v/>
-      </c>
-      <c r="K68" s="7" t="inlineStr">
-        <is>
-          <t>State Name</t>
-        </is>
-      </c>
-      <c r="L68" s="29">
-        <f>C7</f>
+      <c r="B68" s="34" t="inlineStr">
+        <is>
+          <t>Local Effective Rate on the Gain</t>
+        </is>
+      </c>
+      <c r="C68" s="39">
+        <f>IFERROR(C62/C43,0)</f>
+        <v/>
+      </c>
+      <c r="L68" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M68" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N68" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L47)</f>
         <v/>
       </c>
     </row>
     <row r="69" hidden="1" outlineLevel="1">
-      <c r="B69" s="33" t="inlineStr">
-        <is>
-          <t>Ordinary-Taxed Capital Gain / (Loss Deduction, capped)</t>
-        </is>
-      </c>
-      <c r="C69" s="34">
-        <f>IF(C68&lt;=0,MAX(C68,-C62),IF(AND(C66&gt;=0,C67&gt;=0),C66,IF(AND(C66&lt;0,C67&gt;=0),0,IF(AND(C66&gt;=0,C67&lt;0),C68,0))))</f>
-        <v/>
-      </c>
-      <c r="K69" s="7" t="inlineStr">
-        <is>
-          <t>State Code</t>
-        </is>
-      </c>
-      <c r="L69" s="29">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L68,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
+      <c r="L69" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M69" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N69" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L47)</f>
         <v/>
       </c>
     </row>
     <row r="70" hidden="1" outlineLevel="1">
-      <c r="B70" s="33" t="inlineStr">
-        <is>
-          <t>Preferential (LTCG-Rate) Net Capital Gain</t>
-        </is>
-      </c>
-      <c r="C70" s="34">
-        <f>IF(C68&lt;=0,0,IF(AND(C66&gt;=0,C67&gt;=0),C67,IF(AND(C66&lt;0,C67&gt;=0),C68,IF(AND(C66&gt;=0,C67&lt;0),0,0))))</f>
-        <v/>
-      </c>
-      <c r="K70" s="7" t="inlineStr">
-        <is>
-          <t>State Category</t>
-        </is>
-      </c>
-      <c r="L70" s="29">
-        <f>IF(L61="Married Filing Jointly","MFJ","Single")</f>
+      <c r="L70" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M70" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N70" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L47)</f>
         <v/>
       </c>
     </row>
     <row r="71" hidden="1" outlineLevel="1">
-      <c r="B71" s="33" t="inlineStr">
-        <is>
-          <t>Capital Loss Carryforward to Future Years</t>
-        </is>
-      </c>
-      <c r="C71" s="34">
-        <f>IF(C68&lt;=0,C68-MAX(C68,-C62),0)</f>
-        <v/>
-      </c>
-      <c r="K71" s="7" t="inlineStr">
-        <is>
-          <t>State Key</t>
-        </is>
-      </c>
-      <c r="L71" s="29">
-        <f>L69&amp;"|"&amp;L70</f>
+      <c r="L71" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M71" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N71" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L47)</f>
         <v/>
       </c>
     </row>
     <row r="72" hidden="1" outlineLevel="1">
-      <c r="B72" s="33" t="inlineStr">
-        <is>
-          <t>Ordinary Taxable Income Including Gain</t>
-        </is>
-      </c>
-      <c r="C72" s="34">
-        <f>MAX(0,C11+C69)</f>
-        <v/>
-      </c>
-      <c r="K72" s="7" t="inlineStr">
-        <is>
-          <t>State Bracket Row#</t>
-        </is>
-      </c>
-      <c r="L72" s="29">
-        <f>MATCH(L71,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
+      <c r="L72" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M72" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N72" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L47)</f>
         <v/>
       </c>
     </row>
     <row r="73" hidden="1" outlineLevel="1">
-      <c r="B73" s="33" t="inlineStr">
-        <is>
-          <t>Federal Tax on Taxable Income Alone (no gain)</t>
-        </is>
-      </c>
-      <c r="C73" s="34">
-        <f>SUMPRODUCT((C11&gt;$M$76:$M$82)*($L$76:$L$82)*(MIN(C11,$N$76:$N$82)-$M$76:$M$82))</f>
-        <v/>
-      </c>
-      <c r="K73" s="7" t="inlineStr">
-        <is>
-          <t>State Master Row#</t>
-        </is>
-      </c>
-      <c r="L73" s="29">
-        <f>MATCH(L69,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
+      <c r="L73" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M73" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N73" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L47)</f>
         <v/>
       </c>
     </row>
     <row r="74" hidden="1" outlineLevel="1">
-      <c r="B74" s="33" t="inlineStr">
-        <is>
-          <t>Federal Tax on Taxable Income Including Short-Term Gain</t>
-        </is>
-      </c>
-      <c r="C74" s="34">
-        <f>SUMPRODUCT((C72&gt;$M$76:$M$82)*($L$76:$L$82)*(MIN(C72,$N$76:$N$82)-$M$76:$M$82))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" hidden="1" outlineLevel="1">
-      <c r="B75" s="36" t="inlineStr">
-        <is>
-          <t>Federal Tax on Short-Term Gain</t>
-        </is>
-      </c>
-      <c r="C75" s="34">
-        <f>MAX(0,C74-C73)</f>
-        <v/>
-      </c>
-      <c r="K75" s="30" t="inlineStr">
-        <is>
-          <t>Federal Ordinary Brackets</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" hidden="1" outlineLevel="1">
-      <c r="B76" s="36" t="inlineStr">
-        <is>
-          <t>Federal Tax on Long-Term Gain (stacked)</t>
-        </is>
-      </c>
-      <c r="C76" s="34">
-        <f>SUMPRODUCT($L$85:$L$87*(MAX(0,MIN((C72+C70),$N$85:$N$87)-MAX(C72,$M$85:$M$87))))</f>
-        <v/>
-      </c>
-      <c r="L76" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="M76" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="N76" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" hidden="1" outlineLevel="1">
-      <c r="B77" s="33" t="inlineStr">
-        <is>
-          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
-        </is>
-      </c>
-      <c r="C77" s="34">
-        <f>(C11+C61+C69+C70)</f>
-        <v/>
-      </c>
-      <c r="L77" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="M77" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="N77" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78" hidden="1" outlineLevel="1">
-      <c r="B78" s="33" t="inlineStr">
-        <is>
-          <t>Net Investment Income (the modeled capital gain)</t>
-        </is>
-      </c>
-      <c r="C78" s="34">
-        <f>MAX(0,C69+C70)</f>
-        <v/>
-      </c>
-      <c r="L78" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="M78" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="N78" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79" hidden="1" outlineLevel="1">
-      <c r="B79" s="36" t="inlineStr">
-        <is>
-          <t>NIIT</t>
-        </is>
-      </c>
-      <c r="C79" s="34">
-        <f>C64*MIN(C78,MAX(0,C77-C63))</f>
-        <v/>
-      </c>
-      <c r="L79" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="M79" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="N79" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80" hidden="1" outlineLevel="1">
-      <c r="B80" s="33" t="inlineStr">
-        <is>
-          <t>State Taxable Income (gain taxed as ordinary income)</t>
-        </is>
-      </c>
-      <c r="C80" s="34">
-        <f>MAX(0,C11+C69+C70-C65)</f>
-        <v/>
-      </c>
-      <c r="L80" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="M80" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="N80" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" hidden="1" outlineLevel="1">
-      <c r="B81" s="36" t="inlineStr">
-        <is>
-          <t>State Tax</t>
-        </is>
-      </c>
-      <c r="C81" s="34">
-        <f>IF(L69="OTHER",C10*C80,SUMPRODUCT((C80&gt;$M$90:$M$97)*($L$90:$L$97)*(MIN(C80,$N$90:$N$97)-$M$90:$M$97)))</f>
-        <v/>
-      </c>
-      <c r="L81" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="M81" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="N81" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" hidden="1" outlineLevel="1">
-      <c r="B82" s="21" t="inlineStr">
-        <is>
-          <t>Total Estimated Tax</t>
-        </is>
-      </c>
-      <c r="C82" s="37">
-        <f>(C75+C76+C79+C81)</f>
-        <v/>
-      </c>
-      <c r="L82" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="M82" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L64)</f>
-        <v/>
-      </c>
-      <c r="N82" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L64)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83" hidden="1" outlineLevel="1">
-      <c r="B83" s="33" t="inlineStr">
-        <is>
-          <t>Effective Tax Rate on the Gain</t>
-        </is>
-      </c>
-      <c r="C83" s="38">
-        <f>IFERROR(C82/MAX(0.0001,C68),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84" hidden="1" outlineLevel="1">
-      <c r="B84" s="33" t="inlineStr">
-        <is>
-          <t>Marginal LTCG Rate Applied</t>
-        </is>
-      </c>
-      <c r="C84" s="38">
-        <f>IFERROR(INDEX($L$85:$L$87,MATCH(C72,$M$85:$M$87,1)),0)</f>
-        <v/>
-      </c>
-      <c r="K84" s="30" t="inlineStr">
-        <is>
-          <t>LTCG Brackets</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" hidden="1" outlineLevel="1">
-      <c r="B85" s="33" t="inlineStr">
-        <is>
-          <t>State Marginal Tax Rate (on taxable income before any gain)</t>
-        </is>
-      </c>
-      <c r="C85" s="38">
-        <f>IF(L69="OTHER",C10,IFERROR(INDEX($L$90:$L$97,MATCH(MAX(0,C11-C65),$M$90:$M$97,1)),0))</f>
-        <v/>
-      </c>
-      <c r="L85" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L65)</f>
-        <v/>
-      </c>
-      <c r="M85" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L65)</f>
-        <v/>
-      </c>
-      <c r="N85" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L65)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86" hidden="1" outlineLevel="1">
-      <c r="L86" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L65)</f>
-        <v/>
-      </c>
-      <c r="M86" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L65)</f>
-        <v/>
-      </c>
-      <c r="N86" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L65)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87" hidden="1" outlineLevel="1">
-      <c r="L87" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L65)</f>
-        <v/>
-      </c>
-      <c r="M87" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L65)</f>
-        <v/>
-      </c>
-      <c r="N87" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L65)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" hidden="1" outlineLevel="1"/>
-    <row r="89" hidden="1" outlineLevel="1">
-      <c r="K89" s="30" t="inlineStr">
-        <is>
-          <t>State Brackets</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" hidden="1" outlineLevel="1">
-      <c r="L90" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M90" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N90" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" hidden="1" outlineLevel="1">
-      <c r="L91" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M91" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N91" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" hidden="1" outlineLevel="1">
-      <c r="L92" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M92" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N92" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93" hidden="1" outlineLevel="1">
-      <c r="L93" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M93" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N93" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94" hidden="1" outlineLevel="1">
-      <c r="L94" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M94" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N94" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="95" hidden="1" outlineLevel="1">
-      <c r="L95" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M95" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N95" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96" hidden="1" outlineLevel="1">
-      <c r="L96" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M96" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N96" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97" hidden="1" outlineLevel="1">
-      <c r="L97" s="31">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="M97" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L72)</f>
-        <v/>
-      </c>
-      <c r="N97" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L72)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="98" hidden="1" outlineLevel="1"/>
+      <c r="L74" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="M74" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L47)</f>
+        <v/>
+      </c>
+      <c r="N74" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1"/>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="B55:F57"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="B9:F9"/>
+  <mergeCells count="7">
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B18:I19"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B28:I30"/>
+    <mergeCell ref="B32:F32"/>
   </mergeCells>
-  <dataValidations count="3">
-    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="5">
+    <dataValidation sqref="I5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"One year or less,More than a year"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>='Tax Rates &amp; Assumptions'!$B$46:$B$77</formula1>
+    </dataValidation>
+    <dataValidation sqref="I8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Single,Married Filing Jointly,Married Filing Separately,Head of Household"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2024,2025"</formula1>
     </dataValidation>
-    <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Single,Married Filing Jointly,Married Filing Separately,Head of Household"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>='Tax Rates &amp; Assumptions'!$B$46:$B$77</formula1>
+    <dataValidation sqref="F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>='Tax Rates &amp; Assumptions'!$B$148:$B$161</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1901,7 +1790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA160"/>
+  <dimension ref="A1:AA181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -10872,168 +10761,617 @@
         <v>999999999</v>
       </c>
     </row>
+    <row r="146" ht="18" customHeight="1">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>Local / Municipal Tax Table</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="n"/>
+      <c r="C146" s="4" t="n"/>
+      <c r="D146" s="4" t="n"/>
+      <c r="E146" s="4" t="n"/>
+      <c r="F146" s="4" t="n"/>
+      <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="n"/>
+      <c r="I146" s="4" t="n"/>
+      <c r="J146" s="4" t="n"/>
+      <c r="K146" s="4" t="n"/>
+      <c r="L146" s="4" t="n"/>
+      <c r="M146" s="4" t="n"/>
+      <c r="N146" s="4" t="n"/>
+      <c r="O146" s="4" t="n"/>
+      <c r="P146" s="4" t="n"/>
+      <c r="Q146" s="4" t="n"/>
+      <c r="R146" s="4" t="n"/>
+      <c r="S146" s="4" t="n"/>
+      <c r="T146" s="4" t="n"/>
+      <c r="U146" s="4" t="n"/>
+      <c r="V146" s="4" t="n"/>
+      <c r="W146" s="4" t="n"/>
+      <c r="X146" s="4" t="n"/>
+    </row>
     <row r="147">
-      <c r="A147" s="16" t="inlineStr">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>Locality Code</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Locality Name</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="C148" s="12" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="D148" s="14" t="n">
+        <v>0.03648</v>
+      </c>
+      <c r="E148" s="15" t="inlineStr">
+        <is>
+          <t>Approximate blended NYC resident rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="12" t="inlineStr">
+        <is>
+          <t>YONK</t>
+        </is>
+      </c>
+      <c r="B149" s="12" t="inlineStr">
+        <is>
+          <t>Yonkers (NY)</t>
+        </is>
+      </c>
+      <c r="C149" s="12" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="D149" s="14" t="n">
+        <v>0.1675</v>
+      </c>
+      <c r="E149" s="15" t="inlineStr">
+        <is>
+          <t>Resident surcharge as % of NY State tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="inlineStr">
+        <is>
+          <t>PHIL</t>
+        </is>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t>Philadelphia, PA</t>
+        </is>
+      </c>
+      <c r="C150" s="12" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="D150" s="14" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="E150" s="15" t="inlineStr">
+        <is>
+          <t>Philadelphia wage tax (resident).</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="12" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="B151" s="12" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA</t>
+        </is>
+      </c>
+      <c r="C151" s="12" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="D151" s="14" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E151" s="15" t="inlineStr">
+        <is>
+          <t>Local earned income tax (approx.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="B152" s="12" t="inlineStr">
+        <is>
+          <t>Detroit, MI</t>
+        </is>
+      </c>
+      <c r="C152" s="12" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="D152" s="14" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="E152" s="15" t="inlineStr">
+        <is>
+          <t>Detroit resident income tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="12" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="B153" s="12" t="inlineStr">
+        <is>
+          <t>Columbus, OH</t>
+        </is>
+      </c>
+      <c r="C153" s="12" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D153" s="14" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="E153" s="15" t="inlineStr">
+        <is>
+          <t>Ohio municipal income tax (approx.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
+        <is>
+          <t>CIN</t>
+        </is>
+      </c>
+      <c r="B154" s="12" t="inlineStr">
+        <is>
+          <t>Cincinnati, OH</t>
+        </is>
+      </c>
+      <c r="C154" s="12" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D154" s="14" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="E154" s="15" t="inlineStr">
+        <is>
+          <t>Ohio municipal income tax (approx.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="12" t="inlineStr">
+        <is>
+          <t>CLE</t>
+        </is>
+      </c>
+      <c r="B155" s="12" t="inlineStr">
+        <is>
+          <t>Cleveland, OH</t>
+        </is>
+      </c>
+      <c r="C155" s="12" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D155" s="14" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="E155" s="15" t="inlineStr">
+        <is>
+          <t>Ohio municipal income tax (approx.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
+        <is>
+          <t>MDCO</t>
+        </is>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t>Maryland County (avg.)</t>
+        </is>
+      </c>
+      <c r="C156" s="12" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="D156" s="14" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E156" s="15" t="inlineStr">
+        <is>
+          <t>Average MD county piggyback tax as % of state taxable income equivalent (approx.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="12" t="inlineStr">
+        <is>
+          <t>INCO</t>
+        </is>
+      </c>
+      <c r="B157" s="12" t="inlineStr">
+        <is>
+          <t>Indiana County (avg.)</t>
+        </is>
+      </c>
+      <c r="C157" s="12" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D157" s="14" t="n">
+        <v>0.0165</v>
+      </c>
+      <c r="E157" s="15" t="inlineStr">
+        <is>
+          <t>Average Indiana county income tax (approx.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="12" t="inlineStr">
+        <is>
+          <t>KCMO</t>
+        </is>
+      </c>
+      <c r="B158" s="12" t="inlineStr">
+        <is>
+          <t>Kansas City, MO</t>
+        </is>
+      </c>
+      <c r="C158" s="12" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="D158" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E158" s="15" t="inlineStr">
+        <is>
+          <t>Local earnings tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="12" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="B159" s="12" t="inlineStr">
+        <is>
+          <t>St. Louis, MO</t>
+        </is>
+      </c>
+      <c r="C159" s="12" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="D159" s="14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E159" s="15" t="inlineStr">
+        <is>
+          <t>Local earnings tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="12" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="B160" s="12" t="inlineStr">
+        <is>
+          <t>None / Not Applicable</t>
+        </is>
+      </c>
+      <c r="C160" s="12" t="inlineStr"/>
+      <c r="D160" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" s="15" t="inlineStr">
+        <is>
+          <t>No local tax.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="12" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="B161" s="12" t="inlineStr">
+        <is>
+          <t>Other (Manual Entry)</t>
+        </is>
+      </c>
+      <c r="C161" s="12" t="inlineStr"/>
+      <c r="D161" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" s="15" t="inlineStr">
+        <is>
+          <t>Enter a custom local rate on the Inputs tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>Personal Exemption Assumption</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="n"/>
+      <c r="C163" s="4" t="n"/>
+      <c r="D163" s="4" t="n"/>
+      <c r="E163" s="4" t="n"/>
+      <c r="F163" s="4" t="n"/>
+      <c r="G163" s="4" t="n"/>
+      <c r="H163" s="4" t="n"/>
+      <c r="I163" s="4" t="n"/>
+      <c r="J163" s="4" t="n"/>
+      <c r="K163" s="4" t="n"/>
+      <c r="L163" s="4" t="n"/>
+      <c r="M163" s="4" t="n"/>
+      <c r="N163" s="4" t="n"/>
+      <c r="O163" s="4" t="n"/>
+      <c r="P163" s="4" t="n"/>
+      <c r="Q163" s="4" t="n"/>
+      <c r="R163" s="4" t="n"/>
+      <c r="S163" s="4" t="n"/>
+      <c r="T163" s="4" t="n"/>
+      <c r="U163" s="4" t="n"/>
+      <c r="V163" s="4" t="n"/>
+      <c r="W163" s="4" t="n"/>
+      <c r="X163" s="4" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="16" t="inlineStr">
+        <is>
+          <t>Generic State Personal Exemption Amount (per exemption)</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="17" t="inlineStr">
+        <is>
+          <t>Federal personal exemptions are suspended (set to $0) under current law. Most states that still allow a personal exemption use their own amount; this workbook applies one generic per-exemption reduction to state taxable income for simplicity - update the figure above or refine per state as needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="18" t="inlineStr">
         <is>
           <t>DISCLAIMER: Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions.</t>
         </is>
       </c>
-      <c r="B147" s="17" t="n"/>
-      <c r="C147" s="17" t="n"/>
-      <c r="D147" s="17" t="n"/>
-      <c r="E147" s="17" t="n"/>
-      <c r="F147" s="17" t="n"/>
-      <c r="G147" s="17" t="n"/>
-      <c r="H147" s="17" t="n"/>
-      <c r="I147" s="17" t="n"/>
-      <c r="J147" s="17" t="n"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="17" t="n"/>
-      <c r="B148" s="17" t="n"/>
-      <c r="C148" s="17" t="n"/>
-      <c r="D148" s="17" t="n"/>
-      <c r="E148" s="17" t="n"/>
-      <c r="F148" s="17" t="n"/>
-      <c r="G148" s="17" t="n"/>
-      <c r="H148" s="17" t="n"/>
-      <c r="I148" s="17" t="n"/>
-      <c r="J148" s="17" t="n"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="17" t="n"/>
-      <c r="B149" s="17" t="n"/>
-      <c r="C149" s="17" t="n"/>
-      <c r="D149" s="17" t="n"/>
-      <c r="E149" s="17" t="n"/>
-      <c r="F149" s="17" t="n"/>
-      <c r="G149" s="17" t="n"/>
-      <c r="H149" s="17" t="n"/>
-      <c r="I149" s="17" t="n"/>
-      <c r="J149" s="17" t="n"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="17" t="n"/>
-      <c r="B150" s="17" t="n"/>
-      <c r="C150" s="17" t="n"/>
-      <c r="D150" s="17" t="n"/>
-      <c r="E150" s="17" t="n"/>
-      <c r="F150" s="17" t="n"/>
-      <c r="G150" s="17" t="n"/>
-      <c r="H150" s="17" t="n"/>
-      <c r="I150" s="17" t="n"/>
-      <c r="J150" s="17" t="n"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="17" t="n"/>
-      <c r="B151" s="17" t="n"/>
-      <c r="C151" s="17" t="n"/>
-      <c r="D151" s="17" t="n"/>
-      <c r="E151" s="17" t="n"/>
-      <c r="F151" s="17" t="n"/>
-      <c r="G151" s="17" t="n"/>
-      <c r="H151" s="17" t="n"/>
-      <c r="I151" s="17" t="n"/>
-      <c r="J151" s="17" t="n"/>
-    </row>
-    <row r="153" ht="18" customHeight="1">
-      <c r="A153" s="3" t="inlineStr">
+      <c r="B168" s="19" t="n"/>
+      <c r="C168" s="19" t="n"/>
+      <c r="D168" s="19" t="n"/>
+      <c r="E168" s="19" t="n"/>
+      <c r="F168" s="19" t="n"/>
+      <c r="G168" s="19" t="n"/>
+      <c r="H168" s="19" t="n"/>
+      <c r="I168" s="19" t="n"/>
+      <c r="J168" s="19" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="19" t="n"/>
+      <c r="B169" s="19" t="n"/>
+      <c r="C169" s="19" t="n"/>
+      <c r="D169" s="19" t="n"/>
+      <c r="E169" s="19" t="n"/>
+      <c r="F169" s="19" t="n"/>
+      <c r="G169" s="19" t="n"/>
+      <c r="H169" s="19" t="n"/>
+      <c r="I169" s="19" t="n"/>
+      <c r="J169" s="19" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="19" t="n"/>
+      <c r="B170" s="19" t="n"/>
+      <c r="C170" s="19" t="n"/>
+      <c r="D170" s="19" t="n"/>
+      <c r="E170" s="19" t="n"/>
+      <c r="F170" s="19" t="n"/>
+      <c r="G170" s="19" t="n"/>
+      <c r="H170" s="19" t="n"/>
+      <c r="I170" s="19" t="n"/>
+      <c r="J170" s="19" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="19" t="n"/>
+      <c r="B171" s="19" t="n"/>
+      <c r="C171" s="19" t="n"/>
+      <c r="D171" s="19" t="n"/>
+      <c r="E171" s="19" t="n"/>
+      <c r="F171" s="19" t="n"/>
+      <c r="G171" s="19" t="n"/>
+      <c r="H171" s="19" t="n"/>
+      <c r="I171" s="19" t="n"/>
+      <c r="J171" s="19" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="19" t="n"/>
+      <c r="B172" s="19" t="n"/>
+      <c r="C172" s="19" t="n"/>
+      <c r="D172" s="19" t="n"/>
+      <c r="E172" s="19" t="n"/>
+      <c r="F172" s="19" t="n"/>
+      <c r="G172" s="19" t="n"/>
+      <c r="H172" s="19" t="n"/>
+      <c r="I172" s="19" t="n"/>
+      <c r="J172" s="19" t="n"/>
+    </row>
+    <row r="174" ht="18" customHeight="1">
+      <c r="A174" s="3" t="inlineStr">
         <is>
           <t>Key Assumptions</t>
         </is>
       </c>
-      <c r="B153" s="4" t="n"/>
-      <c r="C153" s="4" t="n"/>
-      <c r="D153" s="4" t="n"/>
-      <c r="E153" s="4" t="n"/>
-      <c r="F153" s="4" t="n"/>
-      <c r="G153" s="4" t="n"/>
-      <c r="H153" s="4" t="n"/>
-      <c r="I153" s="4" t="n"/>
-      <c r="J153" s="4" t="n"/>
-      <c r="K153" s="4" t="n"/>
-      <c r="L153" s="4" t="n"/>
-      <c r="M153" s="4" t="n"/>
-      <c r="N153" s="4" t="n"/>
-      <c r="O153" s="4" t="n"/>
-      <c r="P153" s="4" t="n"/>
-      <c r="Q153" s="4" t="n"/>
-      <c r="R153" s="4" t="n"/>
-      <c r="S153" s="4" t="n"/>
-      <c r="T153" s="4" t="n"/>
-      <c r="U153" s="4" t="n"/>
-      <c r="V153" s="4" t="n"/>
-      <c r="W153" s="4" t="n"/>
-      <c r="X153" s="4" t="n"/>
-    </row>
-    <row r="154" ht="40" customHeight="1">
-      <c r="A154" s="18" t="inlineStr">
+      <c r="B174" s="4" t="n"/>
+      <c r="C174" s="4" t="n"/>
+      <c r="D174" s="4" t="n"/>
+      <c r="E174" s="4" t="n"/>
+      <c r="F174" s="4" t="n"/>
+      <c r="G174" s="4" t="n"/>
+      <c r="H174" s="4" t="n"/>
+      <c r="I174" s="4" t="n"/>
+      <c r="J174" s="4" t="n"/>
+      <c r="K174" s="4" t="n"/>
+      <c r="L174" s="4" t="n"/>
+      <c r="M174" s="4" t="n"/>
+      <c r="N174" s="4" t="n"/>
+      <c r="O174" s="4" t="n"/>
+      <c r="P174" s="4" t="n"/>
+      <c r="Q174" s="4" t="n"/>
+      <c r="R174" s="4" t="n"/>
+      <c r="S174" s="4" t="n"/>
+      <c r="T174" s="4" t="n"/>
+      <c r="U174" s="4" t="n"/>
+      <c r="V174" s="4" t="n"/>
+      <c r="W174" s="4" t="n"/>
+      <c r="X174" s="4" t="n"/>
+    </row>
+    <row r="175" ht="40" customHeight="1">
+      <c r="A175" s="20" t="inlineStr">
         <is>
           <t>• Tax Year Coverage: 2024 and 2025. Every bracket, deduction, and threshold used by the calculator lives on this tab; nothing is hardcoded in the formulas on the Capital Gains Tax Estimator tab.</t>
         </is>
       </c>
     </row>
-    <row r="155" ht="40" customHeight="1">
-      <c r="A155" s="18" t="inlineStr">
+    <row r="176" ht="40" customHeight="1">
+      <c r="A176" s="20" t="inlineStr">
         <is>
           <t>• Short-term and long-term gains/losses are netted using standard IRC Sec. 1211/1222 ordering (Form 8949 / Schedule D concepts): a net short-term loss first offsets net long-term gain (and vice versa) before any loss is allowed against ordinary income, capped at the annual limit above (with the remainder carried forward indefinitely). Long-term capital gains are 'stacked' on top of ordinary taxable income when applying the 0%/15%/20% preferential brackets, so they are taxed at the rate(s) that actually apply given the household's total income - not an average rate. Short-term gains are taxed as ordinary income.</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="40" customHeight="1">
-      <c r="A156" s="18" t="inlineStr">
+    <row r="177" ht="40" customHeight="1">
+      <c r="A177" s="20" t="inlineStr">
         <is>
           <t>• The Net Investment Income Tax (3.8%) MAGI thresholds are fixed by statute and have not been inflation-adjusted since enactment (2013). MAGI is approximated as taxable ordinary income plus the net capital gain being modeled.</t>
         </is>
       </c>
     </row>
-    <row r="157" ht="40" customHeight="1">
-      <c r="A157" s="18" t="inlineStr">
+    <row r="178" ht="40" customHeight="1">
+      <c r="A178" s="20" t="inlineStr">
         <is>
           <t>• 31 states plus Washington D.C. are modeled individually (no-tax, flat-tax, and progressive structures), plus a manual-entry option for any other state - not all 50 states are included. State brackets use two filing categories: 'Single' (applied to Single, Married Filing Separately, and Head of Household) and 'MFJ' (applied to Married Filing Jointly).</t>
         </is>
       </c>
     </row>
-    <row r="158" ht="40" customHeight="1">
-      <c r="A158" s="18" t="inlineStr">
+    <row r="179" ht="40" customHeight="1">
+      <c r="A179" s="20" t="inlineStr">
         <is>
           <t>• All states are assumed to tax capital gains as ordinary income (i.e., no separate state preferential capital-gains rate), which is accurate for the large majority of states. State tax uses a state-specific standard deduction where available; it does not model every state's exemption or credit nuance - this is a planning estimate, not a full state tax return.</t>
         </is>
       </c>
     </row>
-    <row r="159" ht="40" customHeight="1">
-      <c r="A159" s="18" t="inlineStr">
+    <row r="180" ht="40" customHeight="1">
+      <c r="A180" s="20" t="inlineStr">
         <is>
           <t>• Tax-loss harvesting losses entered in the What-If section are assumed to be long-term in character (the common case for most portfolios).</t>
         </is>
       </c>
     </row>
-    <row r="160" ht="40" customHeight="1">
-      <c r="A160" s="18" t="inlineStr">
+    <row r="181" ht="40" customHeight="1">
+      <c r="A181" s="20" t="inlineStr">
         <is>
           <t>• This workbook does not model AMT, Qualified Business Income deductions, or every state/local nuance.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="20">
     <mergeCell ref="A79:X79"/>
-    <mergeCell ref="A160:J160"/>
+    <mergeCell ref="A146:X146"/>
+    <mergeCell ref="A181:J181"/>
+    <mergeCell ref="A174:X174"/>
+    <mergeCell ref="A180:J180"/>
+    <mergeCell ref="A37:X37"/>
+    <mergeCell ref="A165:J165"/>
+    <mergeCell ref="A163:X163"/>
+    <mergeCell ref="A26:X26"/>
+    <mergeCell ref="A176:J176"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A153:X153"/>
-    <mergeCell ref="A155:J155"/>
+    <mergeCell ref="A178:J178"/>
     <mergeCell ref="A4:X4"/>
-    <mergeCell ref="A159:J159"/>
-    <mergeCell ref="A26:X26"/>
+    <mergeCell ref="A44:X44"/>
+    <mergeCell ref="A177:J177"/>
+    <mergeCell ref="A168:J172"/>
     <mergeCell ref="A15:X15"/>
-    <mergeCell ref="A158:J158"/>
-    <mergeCell ref="A154:J154"/>
-    <mergeCell ref="A37:X37"/>
-    <mergeCell ref="A147:J151"/>
-    <mergeCell ref="A156:J156"/>
-    <mergeCell ref="A157:J157"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A44:X44"/>
+    <mergeCell ref="A179:J179"/>
+    <mergeCell ref="A175:J175"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace single-sale inputs with 4 direct gain/loss rows
Swapped Initial Value / Sale Value / Length of Ownership for four
explicit inputs: Long-Term Capital Gain, Long-Term Capital Loss,
Short-Term Capital Gain, Short-Term Capital Loss. Engine now nets
short-term against long-term following standard IRC ordering (a net
loss in one category offsets a gain in the other before the $3,000/
$1,500 annual deduction limit applies) rather than assuming one single
holding period. Everything else - Location/Income/Filing Status, the
collapsible Advanced section, the total banner, and the Federal/State/
Local table - is unchanged. Re-verified formula wiring end to end
(structural checks clean; hand-traced against a worked example).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XveA8LngnD1MFNqnzekQW3
</commit_message>
<xml_diff>
--- a/Capital_Gains_Tax_Estimator.xlsx
+++ b/Capital_Gains_Tax_Estimator.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N74"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -748,200 +748,187 @@
     <row r="4">
       <c r="B4" s="23" t="inlineStr">
         <is>
-          <t>Initial Value</t>
+          <t>Long-Term Capital Gain</t>
         </is>
       </c>
       <c r="E4" s="23" t="inlineStr">
         <is>
-          <t>Sale Value</t>
+          <t>Long-Term Capital Loss</t>
         </is>
       </c>
       <c r="H4" s="23" t="inlineStr">
         <is>
-          <t>Length of Ownership</t>
+          <t>Short-Term Capital Gain</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="C5" s="13" t="n">
-        <v>10000</v>
+        <v>50000</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>50000</v>
-      </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>More than a year</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="23" t="inlineStr">
         <is>
+          <t>Short-Term Capital Loss</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
           <t>Location (State)</t>
         </is>
       </c>
-      <c r="E7" s="23" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>Annual Income</t>
         </is>
       </c>
-      <c r="H7" s="23" t="inlineStr">
+    </row>
+    <row r="8">
+      <c r="C8" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>Filing Status</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>New Jersey</t>
-        </is>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>200000</v>
-      </c>
-      <c r="I8" s="12" t="inlineStr">
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>Tax Year</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>Married Filing Jointly</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Tax Year</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="C10" s="12" t="n">
+      <c r="F11" s="12" t="n">
         <v>2025</v>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="24" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>ADVANCED (optional - click the [+] in the row-number margin to expand)</t>
         </is>
       </c>
     </row>
-    <row r="13" hidden="1" outlineLevel="1" collapsed="1">
-      <c r="B13" s="16" t="inlineStr">
+    <row r="14" hidden="1" outlineLevel="1" collapsed="1">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>401(k) Contribution</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>IRA Contribution</t>
         </is>
       </c>
-      <c r="H13" s="16" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>Itemized Deductions</t>
         </is>
       </c>
     </row>
-    <row r="14" hidden="1" outlineLevel="1">
-      <c r="C14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
     <row r="15" hidden="1" outlineLevel="1">
-      <c r="B15" s="16" t="inlineStr">
+      <c r="C15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" hidden="1" outlineLevel="1">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Number of Personal Exemptions (state only)</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Locality / City (optional)</t>
         </is>
       </c>
     </row>
-    <row r="16" hidden="1" outlineLevel="1">
-      <c r="C16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
+    <row r="17" hidden="1" outlineLevel="1">
+      <c r="C17" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>None / Not Applicable</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="25">
-        <f>C63</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1"/>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="25">
+        <f>C65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>YOUR CAPITAL GAINS TAXES</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
-      <c r="H21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Tax Type</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Marginal Tax Rate</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Effective Tax Rate</t>
         </is>
       </c>
-      <c r="H22" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>Tax Amount</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>Federal</t>
-        </is>
-      </c>
-      <c r="D23" s="40">
-        <f>C64</f>
-        <v/>
-      </c>
-      <c r="F23" s="40">
-        <f>C65</f>
-        <v/>
-      </c>
-      <c r="H23" s="41">
-        <f>C56</f>
-        <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="D24" s="40">
@@ -953,830 +940,855 @@
         <v/>
       </c>
       <c r="H24" s="41">
-        <f>C61</f>
+        <f>C58</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="23" t="inlineStr">
         <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="D25" s="40">
+        <f>C68</f>
+        <v/>
+      </c>
+      <c r="F25" s="40">
+        <f>C69</f>
+        <v/>
+      </c>
+      <c r="H25" s="41">
+        <f>C63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="23" t="inlineStr">
+        <is>
           <t>Local</t>
         </is>
       </c>
-      <c r="D25" s="40">
-        <f>C42</f>
-        <v/>
-      </c>
-      <c r="F25" s="40">
-        <f>C68</f>
-        <v/>
-      </c>
-      <c r="H25" s="41">
-        <f>C62</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="26" t="inlineStr">
+      <c r="D26" s="40">
+        <f>C43</f>
+        <v/>
+      </c>
+      <c r="F26" s="40">
+        <f>C70</f>
+        <v/>
+      </c>
+      <c r="H26" s="41">
+        <f>C64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
         </is>
       </c>
-      <c r="H26" s="42">
-        <f>C63</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="27" t="inlineStr">
+      <c r="H27" s="42">
+        <f>C65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>Estimated for financial-planning purposes only. This calculator is not tax, legal, or accounting advice. Actual tax liability may differ based on individual circumstances, deductions, credits, tax elections, state/local rules, and other factors. Consult a qualified tax professional before making tax-related decisions. "Federal" includes the Net Investment Income Tax (3.8%) where applicable.</t>
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30"/>
-    <row r="32">
-      <c r="B32" s="28" t="inlineStr">
+    <row r="31"/>
+    <row r="33">
+      <c r="B33" s="28" t="inlineStr">
         <is>
           <t>Full calculation detail is available below for your advisor. Click the [+] in the row-number margin to expand.</t>
         </is>
       </c>
     </row>
-    <row r="34" hidden="1" outlineLevel="1" collapsed="1">
-      <c r="A34" s="29" t="inlineStr">
+    <row r="35" hidden="1" outlineLevel="1" collapsed="1">
+      <c r="A35" s="29" t="inlineStr">
         <is>
           <t>CALCULATION DETAIL (grouped - click + to expand)</t>
         </is>
       </c>
     </row>
-    <row r="35" hidden="1" outlineLevel="1"/>
-    <row r="36" hidden="1" outlineLevel="1">
-      <c r="B36" s="34" t="inlineStr">
-        <is>
-          <t>Standard Deduction (add-back for MAGI estimate)</t>
-        </is>
-      </c>
-      <c r="C36" s="35">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L42)</f>
-        <v/>
-      </c>
-      <c r="K36" s="7" t="inlineStr">
-        <is>
-          <t>Filing Status</t>
-        </is>
-      </c>
-      <c r="L36" s="30">
-        <f>I8</f>
-        <v/>
-      </c>
-    </row>
+    <row r="36" hidden="1" outlineLevel="1"/>
     <row r="37" hidden="1" outlineLevel="1">
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>Capital Loss Limit vs. Ordinary Income</t>
+          <t>Standard Deduction (add-back for MAGI estimate)</t>
         </is>
       </c>
       <c r="C37" s="35">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L41)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L43)</f>
         <v/>
       </c>
       <c r="K37" s="7" t="inlineStr">
         <is>
-          <t>Tax Year</t>
+          <t>Filing Status</t>
         </is>
       </c>
       <c r="L37" s="30">
-        <f>C10</f>
+        <f>C11</f>
         <v/>
       </c>
     </row>
     <row r="38" hidden="1" outlineLevel="1">
       <c r="B38" s="34" t="inlineStr">
         <is>
-          <t>NIIT Threshold</t>
+          <t>Capital Loss Limit vs. Ordinary Income</t>
         </is>
       </c>
       <c r="C38" s="35">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L41)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!$D$39:$D$42,L42)</f>
         <v/>
       </c>
       <c r="K38" s="7" t="inlineStr">
         <is>
-          <t>Federal Key</t>
+          <t>Tax Year</t>
         </is>
       </c>
       <c r="L38" s="30">
-        <f>L37&amp;"|"&amp;L36</f>
+        <f>F11</f>
         <v/>
       </c>
     </row>
     <row r="39" hidden="1" outlineLevel="1">
       <c r="B39" s="34" t="inlineStr">
         <is>
-          <t>NIIT Rate</t>
-        </is>
-      </c>
-      <c r="C39" s="36">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L41)</f>
+          <t>NIIT Threshold</t>
+        </is>
+      </c>
+      <c r="C39" s="35">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$B$39:$B$42,L42)</f>
         <v/>
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>Fed Bracket Row#</t>
+          <t>Federal Key</t>
         </is>
       </c>
       <c r="L39" s="30">
-        <f>MATCH(L38,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
+        <f>L38&amp;"|"&amp;L37</f>
         <v/>
       </c>
     </row>
     <row r="40" hidden="1" outlineLevel="1">
       <c r="B40" s="34" t="inlineStr">
         <is>
-          <t>State Standard Deduction</t>
-        </is>
-      </c>
-      <c r="C40" s="35">
-        <f>IF(L45="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L48),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L48))</f>
+          <t>NIIT Rate</t>
+        </is>
+      </c>
+      <c r="C40" s="36">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$C$39:$C$42,L42)</f>
         <v/>
       </c>
       <c r="K40" s="7" t="inlineStr">
         <is>
-          <t>LTCG Bracket Row#</t>
+          <t>Fed Bracket Row#</t>
         </is>
       </c>
       <c r="L40" s="30">
-        <f>MATCH(L38,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
+        <f>MATCH(L39,'Tax Rates &amp; Assumptions'!$C$6:$C$13,0)</f>
         <v/>
       </c>
     </row>
     <row r="41" hidden="1" outlineLevel="1">
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>Personal Exemption Amount (per exemption, state)</t>
+          <t>State Standard Deduction</t>
         </is>
       </c>
       <c r="C41" s="35">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$C$164:$C$164,1)</f>
+        <f>IF(L46="MFJ",INDEX('Tax Rates &amp; Assumptions'!$E$46:$E$77,L49),INDEX('Tax Rates &amp; Assumptions'!$D$46:$D$77,L49))</f>
         <v/>
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>Status Row# (NIIT/CapLoss)</t>
+          <t>LTCG Bracket Row#</t>
         </is>
       </c>
       <c r="L41" s="30">
-        <f>MATCH(L36,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
+        <f>MATCH(L39,'Tax Rates &amp; Assumptions'!$C$17:$C$24,0)</f>
         <v/>
       </c>
     </row>
     <row r="42" hidden="1" outlineLevel="1">
       <c r="B42" s="34" t="inlineStr">
         <is>
-          <t>Local Tax Rate</t>
-        </is>
-      </c>
-      <c r="C42" s="36">
-        <f>IF(L50=0,0,INDEX('Tax Rates &amp; Assumptions'!$D$148:$D$161,L50))</f>
+          <t>Personal Exemption Amount (per exemption, state)</t>
+        </is>
+      </c>
+      <c r="C42" s="35">
+        <f>INDEX('Tax Rates &amp; Assumptions'!$C$164:$C$164,1)</f>
         <v/>
       </c>
       <c r="K42" s="7" t="inlineStr">
         <is>
-          <t>StdDed Row#</t>
+          <t>Status Row# (NIIT/CapLoss)</t>
         </is>
       </c>
       <c r="L42" s="30">
-        <f>MATCH(L38,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
+        <f>MATCH(L37,'Tax Rates &amp; Assumptions'!$A$39:$A$42,0)</f>
         <v/>
       </c>
     </row>
     <row r="43" hidden="1" outlineLevel="1">
       <c r="B43" s="34" t="inlineStr">
         <is>
-          <t>Capital Gain / (Loss) on Sale</t>
-        </is>
-      </c>
-      <c r="C43" s="35">
-        <f>(F5-C5)</f>
+          <t>Local Tax Rate</t>
+        </is>
+      </c>
+      <c r="C43" s="36">
+        <f>IF(L51=0,0,INDEX('Tax Rates &amp; Assumptions'!$D$148:$D$161,L51))</f>
         <v/>
       </c>
       <c r="K43" s="7" t="inlineStr">
         <is>
-          <t>State Name</t>
+          <t>StdDed Row#</t>
         </is>
       </c>
       <c r="L43" s="30">
-        <f>C8</f>
+        <f>MATCH(L39,'Tax Rates &amp; Assumptions'!$C$28:$C$35,0)</f>
         <v/>
       </c>
     </row>
     <row r="44" hidden="1" outlineLevel="1">
       <c r="B44" s="34" t="inlineStr">
         <is>
-          <t>Is Long-Term?</t>
+          <t>Net Short-Term Gain / (Loss)</t>
         </is>
       </c>
       <c r="C44" s="35">
-        <f>IF(I5="More than a year",1,0)</f>
+        <f>(I5-C8)</f>
         <v/>
       </c>
       <c r="K44" s="7" t="inlineStr">
         <is>
-          <t>State Code</t>
+          <t>State Name</t>
         </is>
       </c>
       <c r="L44" s="30">
-        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L43,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
+        <f>F8</f>
         <v/>
       </c>
     </row>
     <row r="45" hidden="1" outlineLevel="1">
       <c r="B45" s="34" t="inlineStr">
         <is>
-          <t>Ordinary-Taxed Portion (short-term gain, or loss deduction capped)</t>
+          <t>Net Long-Term Gain / (Loss)</t>
         </is>
       </c>
       <c r="C45" s="35">
-        <f>IF(C43&gt;=0,IF(C44=1,0,C43),MAX(C43,-C37))</f>
+        <f>(C5-F5)</f>
         <v/>
       </c>
       <c r="K45" s="7" t="inlineStr">
         <is>
-          <t>State Category</t>
+          <t>State Code</t>
         </is>
       </c>
       <c r="L45" s="30">
-        <f>IF(L36="Married Filing Jointly","MFJ","Single")</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!$A$46:$A$77,MATCH(L44,'Tax Rates &amp; Assumptions'!$B$46:$B$77,0))</f>
         <v/>
       </c>
     </row>
     <row r="46" hidden="1" outlineLevel="1">
       <c r="B46" s="34" t="inlineStr">
         <is>
-          <t>Preferential-Rate Portion (long-term gain)</t>
+          <t>Combined Net Capital Gain / (Loss)</t>
         </is>
       </c>
       <c r="C46" s="35">
-        <f>IF(C43&gt;=0,IF(C44=1,C43,0),0)</f>
+        <f>(C44+C45)</f>
         <v/>
       </c>
       <c r="K46" s="7" t="inlineStr">
         <is>
-          <t>State Key</t>
+          <t>State Category</t>
         </is>
       </c>
       <c r="L46" s="30">
-        <f>L44&amp;"|"&amp;L45</f>
+        <f>IF(L37="Married Filing Jointly","MFJ","Single")</f>
         <v/>
       </c>
     </row>
     <row r="47" hidden="1" outlineLevel="1">
       <c r="B47" s="34" t="inlineStr">
         <is>
-          <t>Taxable Income Before the Gain</t>
+          <t>Ordinary-Taxed Portion (net short-term gain, or loss deduction capped)</t>
         </is>
       </c>
       <c r="C47" s="35">
-        <f>MAX(0,F8-C14-F14-MAX(I14,INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L42)))</f>
+        <f>IF(C46&lt;=0,MAX(C46,-C38),IF(AND(C44&gt;=0,C45&gt;=0),C44,IF(AND(C44&lt;0,C45&gt;=0),0,IF(AND(C44&gt;=0,C45&lt;0),C46,0))))</f>
         <v/>
       </c>
       <c r="K47" s="7" t="inlineStr">
         <is>
-          <t>State Bracket Row#</t>
+          <t>State Key</t>
         </is>
       </c>
       <c r="L47" s="30">
-        <f>MATCH(L46,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
+        <f>L45&amp;"|"&amp;L46</f>
         <v/>
       </c>
     </row>
     <row r="48" hidden="1" outlineLevel="1">
       <c r="B48" s="34" t="inlineStr">
         <is>
-          <t>Taxable Income Including the Gain</t>
+          <t>Preferential-Rate Portion (net long-term gain)</t>
         </is>
       </c>
       <c r="C48" s="35">
-        <f>MAX(0,C47+C45)</f>
+        <f>IF(C46&lt;=0,0,IF(AND(C44&gt;=0,C45&gt;=0),C45,IF(AND(C44&lt;0,C45&gt;=0),C46,IF(AND(C44&gt;=0,C45&lt;0),0,0))))</f>
         <v/>
       </c>
       <c r="K48" s="7" t="inlineStr">
         <is>
-          <t>State Master Row#</t>
+          <t>State Bracket Row#</t>
         </is>
       </c>
       <c r="L48" s="30">
-        <f>MATCH(L44,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
+        <f>MATCH(L47,'Tax Rates &amp; Assumptions'!$C$81:$C$144,0)</f>
         <v/>
       </c>
     </row>
     <row r="49" hidden="1" outlineLevel="1">
       <c r="B49" s="34" t="inlineStr">
         <is>
-          <t>Federal Tax on Income Alone (no gain)</t>
+          <t>Taxable Income Before the Gain</t>
         </is>
       </c>
       <c r="C49" s="35">
-        <f>SUMPRODUCT((C47&gt;$M$53:$M$59)*($L$53:$L$59)*(MIN(C47,$N$53:$N$59)-$M$53:$M$59))</f>
+        <f>MAX(0,I8-C15-F15-MAX(I15,INDEX('Tax Rates &amp; Assumptions'!$D$28:$D$35,L43)))</f>
         <v/>
       </c>
       <c r="K49" s="7" t="inlineStr">
         <is>
-          <t>Locality Name</t>
+          <t>State Master Row#</t>
         </is>
       </c>
       <c r="L49" s="30">
-        <f>F16</f>
+        <f>MATCH(L45,'Tax Rates &amp; Assumptions'!$A$46:$A$77,0)</f>
         <v/>
       </c>
     </row>
     <row r="50" hidden="1" outlineLevel="1">
       <c r="B50" s="34" t="inlineStr">
         <is>
-          <t>Federal Tax on Income Including the Gain</t>
+          <t>Taxable Income Including the Gain</t>
         </is>
       </c>
       <c r="C50" s="35">
-        <f>SUMPRODUCT((C48&gt;$M$53:$M$59)*($L$53:$L$59)*(MIN(C48,$N$53:$N$59)-$M$53:$M$59))</f>
+        <f>MAX(0,C49+C47)</f>
         <v/>
       </c>
       <c r="K50" s="7" t="inlineStr">
         <is>
-          <t>Locality Row#</t>
+          <t>Locality Name</t>
         </is>
       </c>
       <c r="L50" s="30">
-        <f>IFERROR(MATCH(L49,'Tax Rates &amp; Assumptions'!$B$148:$B$161,0),0)</f>
+        <f>F17</f>
         <v/>
       </c>
     </row>
     <row r="51" hidden="1" outlineLevel="1">
       <c r="B51" s="34" t="inlineStr">
         <is>
-          <t>Federal Tax on Ordinary Portion of the Gain</t>
+          <t>Federal Tax on Income Alone (no gain)</t>
         </is>
       </c>
       <c r="C51" s="35">
-        <f>C50-C49</f>
+        <f>SUMPRODUCT((C49&gt;$M$54:$M$60)*($L$54:$L$60)*(MIN(C49,$N$54:$N$60)-$M$54:$M$60))</f>
+        <v/>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>Locality Row#</t>
+        </is>
+      </c>
+      <c r="L51" s="30">
+        <f>IFERROR(MATCH(L50,'Tax Rates &amp; Assumptions'!$B$148:$B$161,0),0)</f>
         <v/>
       </c>
     </row>
     <row r="52" hidden="1" outlineLevel="1">
       <c r="B52" s="34" t="inlineStr">
         <is>
-          <t>Federal Tax on Preferential (Long-Term) Portion (stacked)</t>
+          <t>Federal Tax on Income Including the Gain</t>
         </is>
       </c>
       <c r="C52" s="35">
-        <f>SUMPRODUCT($L$62:$L$64*(MAX(0,MIN((C48+C46),$N$62:$N$64)-MAX(C48,$M$62:$M$64))))</f>
-        <v/>
-      </c>
-      <c r="K52" s="31" t="inlineStr">
-        <is>
-          <t>Federal Ordinary Brackets</t>
-        </is>
+        <f>SUMPRODUCT((C50&gt;$M$54:$M$60)*($L$54:$L$60)*(MIN(C50,$N$54:$N$60)-$M$54:$M$60))</f>
+        <v/>
       </c>
     </row>
     <row r="53" hidden="1" outlineLevel="1">
       <c r="B53" s="34" t="inlineStr">
         <is>
-          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
+          <t>Federal Tax on Ordinary Portion of the Gain</t>
         </is>
       </c>
       <c r="C53" s="35">
-        <f>(C47+C36+C45+C46)</f>
-        <v/>
-      </c>
-      <c r="L53" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L39)</f>
-        <v/>
-      </c>
-      <c r="M53" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L39)</f>
-        <v/>
-      </c>
-      <c r="N53" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L39)</f>
-        <v/>
+        <f>C52-C51</f>
+        <v/>
+      </c>
+      <c r="K53" s="31" t="inlineStr">
+        <is>
+          <t>Federal Ordinary Brackets</t>
+        </is>
       </c>
     </row>
     <row r="54" hidden="1" outlineLevel="1">
       <c r="B54" s="34" t="inlineStr">
         <is>
-          <t>Net Investment Income (the modeled gain)</t>
+          <t>Federal Tax on Preferential (Long-Term) Portion (stacked)</t>
         </is>
       </c>
       <c r="C54" s="35">
-        <f>MAX(0,C45+C46)</f>
+        <f>SUMPRODUCT($L$63:$L$65*(MAX(0,MIN((C50+C48),$N$63:$N$65)-MAX(C50,$M$63:$M$65))))</f>
         <v/>
       </c>
       <c r="L54" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$6:D$1005,L40)</f>
         <v/>
       </c>
       <c r="M54" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$6:E$1005,L40)</f>
         <v/>
       </c>
       <c r="N54" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$6:F$1005,L40)</f>
         <v/>
       </c>
     </row>
     <row r="55" hidden="1" outlineLevel="1">
       <c r="B55" s="34" t="inlineStr">
         <is>
-          <t>NIIT</t>
+          <t>MAGI Estimate (Taxable Income + Std. Ded. Add-Back + Net Gain)</t>
         </is>
       </c>
       <c r="C55" s="35">
-        <f>C39*MIN(C54,MAX(0,C53-C38))</f>
+        <f>(C49+C37+C47+C48)</f>
         <v/>
       </c>
       <c r="L55" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$6:G$1005,L40)</f>
         <v/>
       </c>
       <c r="M55" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$6:H$1005,L40)</f>
         <v/>
       </c>
       <c r="N55" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$6:I$1005,L40)</f>
         <v/>
       </c>
     </row>
     <row r="56" hidden="1" outlineLevel="1">
-      <c r="B56" s="37" t="inlineStr">
-        <is>
-          <t>Total Federal Tax From the Gain (incl. NIIT)</t>
+      <c r="B56" s="34" t="inlineStr">
+        <is>
+          <t>Net Investment Income (the modeled gain)</t>
         </is>
       </c>
       <c r="C56" s="35">
-        <f>(C51+C52+C55)</f>
+        <f>MAX(0,C47+C48)</f>
         <v/>
       </c>
       <c r="L56" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$6:J$1005,L40)</f>
         <v/>
       </c>
       <c r="M56" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$6:K$1005,L40)</f>
         <v/>
       </c>
       <c r="N56" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$6:L$1005,L40)</f>
         <v/>
       </c>
     </row>
     <row r="57" hidden="1" outlineLevel="1">
       <c r="B57" s="34" t="inlineStr">
         <is>
-          <t>State Taxable Income Before the Gain</t>
+          <t>NIIT</t>
         </is>
       </c>
       <c r="C57" s="35">
-        <f>MAX(0,C47-C40-C16*C41)</f>
+        <f>C40*MIN(C56,MAX(0,C55-C39))</f>
         <v/>
       </c>
       <c r="L57" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$6:M$1005,L40)</f>
         <v/>
       </c>
       <c r="M57" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$6:N$1005,L40)</f>
         <v/>
       </c>
       <c r="N57" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$6:O$1005,L40)</f>
         <v/>
       </c>
     </row>
     <row r="58" hidden="1" outlineLevel="1">
-      <c r="B58" s="34" t="inlineStr">
-        <is>
-          <t>State Taxable Income Including the Gain</t>
+      <c r="B58" s="37" t="inlineStr">
+        <is>
+          <t>Total Federal Tax From the Gain (incl. NIIT)</t>
         </is>
       </c>
       <c r="C58" s="35">
-        <f>MAX(0,C47+C45+C46-C40-C16*C41)</f>
+        <f>(C53+C54+C57)</f>
         <v/>
       </c>
       <c r="L58" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$6:P$1005,L40)</f>
         <v/>
       </c>
       <c r="M58" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$6:Q$1005,L40)</f>
         <v/>
       </c>
       <c r="N58" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$6:R$1005,L40)</f>
         <v/>
       </c>
     </row>
     <row r="59" hidden="1" outlineLevel="1">
       <c r="B59" s="34" t="inlineStr">
         <is>
-          <t>State Tax on Income Alone</t>
+          <t>State Taxable Income Before the Gain</t>
         </is>
       </c>
       <c r="C59" s="35">
-        <f>IF(L44="OTHER",0,SUMPRODUCT((C57&gt;$M$67:$M$74)*($L$67:$L$74)*(MIN(C57,$N$67:$N$74)-$M$67:$M$74)))</f>
+        <f>MAX(0,C49-C41-C17*C42)</f>
         <v/>
       </c>
       <c r="L59" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$6:S$1005,L40)</f>
         <v/>
       </c>
       <c r="M59" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$6:T$1005,L40)</f>
         <v/>
       </c>
       <c r="N59" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L39)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$6:U$1005,L40)</f>
         <v/>
       </c>
     </row>
     <row r="60" hidden="1" outlineLevel="1">
       <c r="B60" s="34" t="inlineStr">
         <is>
+          <t>State Taxable Income Including the Gain</t>
+        </is>
+      </c>
+      <c r="C60" s="35">
+        <f>MAX(0,C49+C47+C48-C41-C17*C42)</f>
+        <v/>
+      </c>
+      <c r="L60" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$6:V$1005,L40)</f>
+        <v/>
+      </c>
+      <c r="M60" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$6:W$1005,L40)</f>
+        <v/>
+      </c>
+      <c r="N60" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$6:X$1005,L40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" hidden="1" outlineLevel="1">
+      <c r="B61" s="34" t="inlineStr">
+        <is>
+          <t>State Tax on Income Alone</t>
+        </is>
+      </c>
+      <c r="C61" s="35">
+        <f>IF(L45="OTHER",0,SUMPRODUCT((C59&gt;$M$68:$M$75)*($L$68:$L$75)*(MIN(C59,$N$68:$N$75)-$M$68:$M$75)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" hidden="1" outlineLevel="1">
+      <c r="B62" s="34" t="inlineStr">
+        <is>
           <t>State Tax on Income Including the Gain</t>
         </is>
       </c>
-      <c r="C60" s="35">
-        <f>IF(L44="OTHER",0,SUMPRODUCT((C58&gt;$M$67:$M$74)*($L$67:$L$74)*(MIN(C58,$N$67:$N$74)-$M$67:$M$74)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61" hidden="1" outlineLevel="1">
-      <c r="B61" s="37" t="inlineStr">
+      <c r="C62" s="35">
+        <f>IF(L45="OTHER",0,SUMPRODUCT((C60&gt;$M$68:$M$75)*($L$68:$L$75)*(MIN(C60,$N$68:$N$75)-$M$68:$M$75)))</f>
+        <v/>
+      </c>
+      <c r="K62" s="31" t="inlineStr">
+        <is>
+          <t>LTCG Brackets</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1">
+      <c r="B63" s="37" t="inlineStr">
         <is>
           <t>State Tax From the Gain</t>
         </is>
       </c>
-      <c r="C61" s="35">
-        <f>(C60-C59)</f>
-        <v/>
-      </c>
-      <c r="K61" s="31" t="inlineStr">
-        <is>
-          <t>LTCG Brackets</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" hidden="1" outlineLevel="1">
-      <c r="B62" s="37" t="inlineStr">
+      <c r="C63" s="35">
+        <f>(C62-C61)</f>
+        <v/>
+      </c>
+      <c r="L63" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L41)</f>
+        <v/>
+      </c>
+      <c r="M63" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L41)</f>
+        <v/>
+      </c>
+      <c r="N63" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" hidden="1" outlineLevel="1">
+      <c r="B64" s="37" t="inlineStr">
         <is>
           <t>Local Tax From the Gain</t>
         </is>
       </c>
-      <c r="C62" s="35">
-        <f>C42*MAX(0,C43)</f>
-        <v/>
-      </c>
-      <c r="L62" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$17:D$1016,L40)</f>
-        <v/>
-      </c>
-      <c r="M62" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$17:E$1016,L40)</f>
-        <v/>
-      </c>
-      <c r="N62" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$17:F$1016,L40)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" hidden="1" outlineLevel="1">
-      <c r="B63" s="23" t="inlineStr">
+      <c r="C64" s="35">
+        <f>C43*MAX(0,C46)</f>
+        <v/>
+      </c>
+      <c r="L64" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L41)</f>
+        <v/>
+      </c>
+      <c r="M64" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L41)</f>
+        <v/>
+      </c>
+      <c r="N64" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" hidden="1" outlineLevel="1">
+      <c r="B65" s="23" t="inlineStr">
         <is>
           <t>Total Estimated Tax</t>
         </is>
       </c>
-      <c r="C63" s="38">
-        <f>(C56+C61+C62)</f>
-        <v/>
-      </c>
-      <c r="L63" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$17:G$1016,L40)</f>
-        <v/>
-      </c>
-      <c r="M63" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$17:H$1016,L40)</f>
-        <v/>
-      </c>
-      <c r="N63" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$17:I$1016,L40)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64" hidden="1" outlineLevel="1">
-      <c r="B64" s="34" t="inlineStr">
-        <is>
-          <t>Federal Marginal Rate Applied to the Gain</t>
-        </is>
-      </c>
-      <c r="C64" s="39">
-        <f>IF(AND(C43&gt;=0,C44=1),IFERROR(INDEX($L$62:$L$64,MATCH(C48,$M$62:$M$64,1)),0),IFERROR(INDEX($L$53:$L$59,MATCH(C48,$M$53:$M$59,1)),0))</f>
-        <v/>
-      </c>
-      <c r="L64" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L40)</f>
-        <v/>
-      </c>
-      <c r="M64" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L40)</f>
-        <v/>
-      </c>
-      <c r="N64" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L40)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65" hidden="1" outlineLevel="1">
-      <c r="B65" s="34" t="inlineStr">
-        <is>
-          <t>Federal Effective Rate on the Gain</t>
-        </is>
-      </c>
-      <c r="C65" s="39">
-        <f>IFERROR(C56/C43,0)</f>
+      <c r="C65" s="38">
+        <f>(C58+C63+C64)</f>
+        <v/>
+      </c>
+      <c r="L65" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$17:J$1016,L41)</f>
+        <v/>
+      </c>
+      <c r="M65" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$17:K$1016,L41)</f>
+        <v/>
+      </c>
+      <c r="N65" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$17:L$1016,L41)</f>
         <v/>
       </c>
     </row>
     <row r="66" hidden="1" outlineLevel="1">
       <c r="B66" s="34" t="inlineStr">
         <is>
-          <t>State Marginal Rate Applied to the Gain</t>
+          <t>Federal Marginal Rate Applied to the Gain</t>
         </is>
       </c>
       <c r="C66" s="39">
-        <f>IF(L44="OTHER",0,IFERROR(INDEX($L$67:$L$74,MATCH(C58,$M$67:$M$74,1)),0))</f>
-        <v/>
-      </c>
-      <c r="K66" s="31" t="inlineStr">
-        <is>
-          <t>State Brackets</t>
-        </is>
+        <f>IF(C48&gt;0,IFERROR(INDEX($L$63:$L$65,MATCH((C50+C48),$M$63:$M$65,1)),0),IFERROR(INDEX($L$54:$L$60,MATCH(C50,$M$54:$M$60,1)),0))</f>
+        <v/>
       </c>
     </row>
     <row r="67" hidden="1" outlineLevel="1">
       <c r="B67" s="34" t="inlineStr">
         <is>
-          <t>State Effective Rate on the Gain</t>
+          <t>Federal Effective Rate on the Gain</t>
         </is>
       </c>
       <c r="C67" s="39">
-        <f>IFERROR(C61/C43,0)</f>
-        <v/>
-      </c>
-      <c r="L67" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L47)</f>
-        <v/>
-      </c>
-      <c r="M67" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L47)</f>
-        <v/>
-      </c>
-      <c r="N67" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L47)</f>
-        <v/>
+        <f>IFERROR(C58/C46,0)</f>
+        <v/>
+      </c>
+      <c r="K67" s="31" t="inlineStr">
+        <is>
+          <t>State Brackets</t>
+        </is>
       </c>
     </row>
     <row r="68" hidden="1" outlineLevel="1">
       <c r="B68" s="34" t="inlineStr">
         <is>
+          <t>State Marginal Rate Applied to the Gain</t>
+        </is>
+      </c>
+      <c r="C68" s="39">
+        <f>IF(L45="OTHER",0,IFERROR(INDEX($L$68:$L$75,MATCH(C60,$M$68:$M$75,1)),0))</f>
+        <v/>
+      </c>
+      <c r="L68" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!D$81:D$1080,L48)</f>
+        <v/>
+      </c>
+      <c r="M68" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!E$81:E$1080,L48)</f>
+        <v/>
+      </c>
+      <c r="N68" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!F$81:F$1080,L48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" hidden="1" outlineLevel="1">
+      <c r="B69" s="34" t="inlineStr">
+        <is>
+          <t>State Effective Rate on the Gain</t>
+        </is>
+      </c>
+      <c r="C69" s="39">
+        <f>IFERROR(C63/C46,0)</f>
+        <v/>
+      </c>
+      <c r="L69" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L48)</f>
+        <v/>
+      </c>
+      <c r="M69" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L48)</f>
+        <v/>
+      </c>
+      <c r="N69" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1">
+      <c r="B70" s="34" t="inlineStr">
+        <is>
           <t>Local Effective Rate on the Gain</t>
         </is>
       </c>
-      <c r="C68" s="39">
-        <f>IFERROR(C62/C43,0)</f>
-        <v/>
-      </c>
-      <c r="L68" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!G$81:G$1080,L47)</f>
-        <v/>
-      </c>
-      <c r="M68" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!H$81:H$1080,L47)</f>
-        <v/>
-      </c>
-      <c r="N68" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!I$81:I$1080,L47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" hidden="1" outlineLevel="1">
-      <c r="L69" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L47)</f>
-        <v/>
-      </c>
-      <c r="M69" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L47)</f>
-        <v/>
-      </c>
-      <c r="N69" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70" hidden="1" outlineLevel="1">
+      <c r="C70" s="39">
+        <f>IFERROR(C64/C46,0)</f>
+        <v/>
+      </c>
       <c r="L70" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!J$81:J$1080,L48)</f>
         <v/>
       </c>
       <c r="M70" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!K$81:K$1080,L48)</f>
         <v/>
       </c>
       <c r="N70" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!L$81:L$1080,L48)</f>
         <v/>
       </c>
     </row>
     <row r="71" hidden="1" outlineLevel="1">
       <c r="L71" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!M$81:M$1080,L48)</f>
         <v/>
       </c>
       <c r="M71" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!N$81:N$1080,L48)</f>
         <v/>
       </c>
       <c r="N71" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!O$81:O$1080,L48)</f>
         <v/>
       </c>
     </row>
     <row r="72" hidden="1" outlineLevel="1">
       <c r="L72" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!P$81:P$1080,L48)</f>
         <v/>
       </c>
       <c r="M72" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!Q$81:Q$1080,L48)</f>
         <v/>
       </c>
       <c r="N72" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!R$81:R$1080,L48)</f>
         <v/>
       </c>
     </row>
     <row r="73" hidden="1" outlineLevel="1">
       <c r="L73" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!S$81:S$1080,L48)</f>
         <v/>
       </c>
       <c r="M73" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!T$81:T$1080,L48)</f>
         <v/>
       </c>
       <c r="N73" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!U$81:U$1080,L48)</f>
         <v/>
       </c>
     </row>
     <row r="74" hidden="1" outlineLevel="1">
       <c r="L74" s="32">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!V$81:V$1080,L48)</f>
         <v/>
       </c>
       <c r="M74" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L47)</f>
+        <f>INDEX('Tax Rates &amp; Assumptions'!W$81:W$1080,L48)</f>
         <v/>
       </c>
       <c r="N74" s="33">
-        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75" hidden="1" outlineLevel="1"/>
+        <f>INDEX('Tax Rates &amp; Assumptions'!X$81:X$1080,L48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1">
+      <c r="L75" s="32">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Y$81:Y$1080,L48)</f>
+        <v/>
+      </c>
+      <c r="M75" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!Z$81:Z$1080,L48)</f>
+        <v/>
+      </c>
+      <c r="N75" s="33">
+        <f>INDEX('Tax Rates &amp; Assumptions'!AA$81:AA$1080,L48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" hidden="1" outlineLevel="1"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B18:I19"/>
-    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="B13:I13"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="B33:F33"/>
+    <mergeCell ref="B29:I31"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B28:I30"/>
-    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B19:I20"/>
+    <mergeCell ref="A22:H22"/>
   </mergeCells>
-  <dataValidations count="5">
-    <dataValidation sqref="I5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"One year or less,More than a year"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="F8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>='Tax Rates &amp; Assumptions'!$B$46:$B$77</formula1>
     </dataValidation>
-    <dataValidation sqref="I8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Single,Married Filing Jointly,Married Filing Separately,Head of Household"</formula1>
     </dataValidation>
-    <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2024,2025"</formula1>
     </dataValidation>
-    <dataValidation sqref="F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>='Tax Rates &amp; Assumptions'!$B$148:$B$161</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>